<commit_message>
add: folder type field
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -9611,6 +9611,12 @@
   </si>
   <si>
     <t>montagne</t>
+  </si>
+  <si>
+    <t>nomenclature</t>
+  </si>
+  <si>
+    <t>domaine</t>
   </si>
 </sst>
 </file>
@@ -77522,6 +77528,466 @@
         <v>151</v>
       </c>
     </row>
+    <row r="3710">
+      <c r="A3710">
+        <v>1769079525</v>
+      </c>
+      <c r="B3710" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3710" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3710" t="s">
+        <v>155</v>
+      </c>
+      <c r="F3710" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3710" t="s">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="3711">
+      <c r="A3711">
+        <v>1769079525</v>
+      </c>
+      <c r="B3711" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3711" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3711" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3711" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3711" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3712">
+      <c r="A3712">
+        <v>1769079525</v>
+      </c>
+      <c r="B3712" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3712" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3712" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3712" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3712" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3713">
+      <c r="A3713">
+        <v>1769079525</v>
+      </c>
+      <c r="B3713" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3713" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3713" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3713" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3713" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3714">
+      <c r="A3714">
+        <v>1769079525</v>
+      </c>
+      <c r="B3714" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3714" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3714" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3714" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3714" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3715">
+      <c r="A3715">
+        <v>1769079525</v>
+      </c>
+      <c r="B3715" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3715" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3715" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3715" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3715" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3716">
+      <c r="A3716">
+        <v>1769079525</v>
+      </c>
+      <c r="B3716" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3716" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3716" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3716" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3716" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3717">
+      <c r="A3717">
+        <v>1769079525</v>
+      </c>
+      <c r="B3717" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3717" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3717" t="s">
+        <v>162</v>
+      </c>
+      <c r="F3717" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3717" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3718">
+      <c r="A3718">
+        <v>1769079525</v>
+      </c>
+      <c r="B3718" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3718" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3718" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3718" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3718" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3719">
+      <c r="A3719">
+        <v>1769079525</v>
+      </c>
+      <c r="B3719" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3719" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3719" t="s">
+        <v>164</v>
+      </c>
+      <c r="F3719" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3719" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3720">
+      <c r="A3720">
+        <v>1769079525</v>
+      </c>
+      <c r="B3720" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3720" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3720" t="s">
+        <v>165</v>
+      </c>
+      <c r="F3720" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3720" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3721">
+      <c r="A3721">
+        <v>1769079525</v>
+      </c>
+      <c r="B3721" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3721" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3721" t="s">
+        <v>166</v>
+      </c>
+      <c r="F3721" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3721" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3722">
+      <c r="A3722">
+        <v>1769079525</v>
+      </c>
+      <c r="B3722" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3722" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3722" t="s">
+        <v>167</v>
+      </c>
+      <c r="F3722" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3722" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3723">
+      <c r="A3723">
+        <v>1769079525</v>
+      </c>
+      <c r="B3723" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3723" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3723" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3723" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3723" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3724">
+      <c r="A3724">
+        <v>1769079525</v>
+      </c>
+      <c r="B3724" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3724" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3724" t="s">
+        <v>168</v>
+      </c>
+      <c r="F3724" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3724" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3725">
+      <c r="A3725">
+        <v>1769079525</v>
+      </c>
+      <c r="B3725" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3725" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3725" t="s">
+        <v>169</v>
+      </c>
+      <c r="F3725" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3725" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3726">
+      <c r="A3726">
+        <v>1769079525</v>
+      </c>
+      <c r="B3726" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3726" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3726" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3726" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3726" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3727">
+      <c r="A3727">
+        <v>1769079525</v>
+      </c>
+      <c r="B3727" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3727" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3727" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3727" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3727" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3728">
+      <c r="A3728">
+        <v>1769079525</v>
+      </c>
+      <c r="B3728" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3728" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3728" t="s">
+        <v>172</v>
+      </c>
+      <c r="F3728" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3728" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3729">
+      <c r="A3729">
+        <v>1769079525</v>
+      </c>
+      <c r="B3729" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3729" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3729" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3729" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3729" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3730">
+      <c r="A3730">
+        <v>1769079525</v>
+      </c>
+      <c r="B3730" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3730" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3730" t="s">
+        <v>174</v>
+      </c>
+      <c r="F3730" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3730" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3731">
+      <c r="A3731">
+        <v>1769079525</v>
+      </c>
+      <c r="B3731" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3731" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3731" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3731" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3731" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3732">
+      <c r="A3732">
+        <v>1769079525</v>
+      </c>
+      <c r="B3732" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3732" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3732" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3732" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3732" t="s">
+        <v>3201</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add: folder type field (#86)
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -9611,6 +9611,12 @@
   </si>
   <si>
     <t>montagne</t>
+  </si>
+  <si>
+    <t>nomenclature</t>
+  </si>
+  <si>
+    <t>domaine</t>
   </si>
 </sst>
 </file>
@@ -77522,6 +77528,466 @@
         <v>151</v>
       </c>
     </row>
+    <row r="3710">
+      <c r="A3710">
+        <v>1769079525</v>
+      </c>
+      <c r="B3710" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3710" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3710" t="s">
+        <v>155</v>
+      </c>
+      <c r="F3710" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3710" t="s">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="3711">
+      <c r="A3711">
+        <v>1769079525</v>
+      </c>
+      <c r="B3711" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3711" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3711" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3711" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3711" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3712">
+      <c r="A3712">
+        <v>1769079525</v>
+      </c>
+      <c r="B3712" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3712" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3712" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3712" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3712" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3713">
+      <c r="A3713">
+        <v>1769079525</v>
+      </c>
+      <c r="B3713" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3713" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3713" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3713" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3713" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3714">
+      <c r="A3714">
+        <v>1769079525</v>
+      </c>
+      <c r="B3714" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3714" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3714" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3714" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3714" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3715">
+      <c r="A3715">
+        <v>1769079525</v>
+      </c>
+      <c r="B3715" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3715" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3715" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3715" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3715" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3716">
+      <c r="A3716">
+        <v>1769079525</v>
+      </c>
+      <c r="B3716" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3716" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3716" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3716" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3716" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3717">
+      <c r="A3717">
+        <v>1769079525</v>
+      </c>
+      <c r="B3717" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3717" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3717" t="s">
+        <v>162</v>
+      </c>
+      <c r="F3717" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3717" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3718">
+      <c r="A3718">
+        <v>1769079525</v>
+      </c>
+      <c r="B3718" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3718" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3718" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3718" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3718" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3719">
+      <c r="A3719">
+        <v>1769079525</v>
+      </c>
+      <c r="B3719" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3719" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3719" t="s">
+        <v>164</v>
+      </c>
+      <c r="F3719" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3719" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3720">
+      <c r="A3720">
+        <v>1769079525</v>
+      </c>
+      <c r="B3720" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3720" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3720" t="s">
+        <v>165</v>
+      </c>
+      <c r="F3720" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3720" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3721">
+      <c r="A3721">
+        <v>1769079525</v>
+      </c>
+      <c r="B3721" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3721" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3721" t="s">
+        <v>166</v>
+      </c>
+      <c r="F3721" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3721" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3722">
+      <c r="A3722">
+        <v>1769079525</v>
+      </c>
+      <c r="B3722" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3722" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3722" t="s">
+        <v>167</v>
+      </c>
+      <c r="F3722" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3722" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3723">
+      <c r="A3723">
+        <v>1769079525</v>
+      </c>
+      <c r="B3723" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3723" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3723" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3723" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3723" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3724">
+      <c r="A3724">
+        <v>1769079525</v>
+      </c>
+      <c r="B3724" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3724" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3724" t="s">
+        <v>168</v>
+      </c>
+      <c r="F3724" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3724" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3725">
+      <c r="A3725">
+        <v>1769079525</v>
+      </c>
+      <c r="B3725" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3725" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3725" t="s">
+        <v>169</v>
+      </c>
+      <c r="F3725" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3725" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3726">
+      <c r="A3726">
+        <v>1769079525</v>
+      </c>
+      <c r="B3726" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3726" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3726" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3726" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3726" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3727">
+      <c r="A3727">
+        <v>1769079525</v>
+      </c>
+      <c r="B3727" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3727" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3727" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3727" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3727" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3728">
+      <c r="A3728">
+        <v>1769079525</v>
+      </c>
+      <c r="B3728" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3728" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3728" t="s">
+        <v>172</v>
+      </c>
+      <c r="F3728" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3728" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3729">
+      <c r="A3729">
+        <v>1769079525</v>
+      </c>
+      <c r="B3729" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3729" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3729" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3729" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3729" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3730">
+      <c r="A3730">
+        <v>1769079525</v>
+      </c>
+      <c r="B3730" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3730" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3730" t="s">
+        <v>174</v>
+      </c>
+      <c r="F3730" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3730" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3731">
+      <c r="A3731">
+        <v>1769079525</v>
+      </c>
+      <c r="B3731" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3731" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3731" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3731" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3731" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="3732">
+      <c r="A3732">
+        <v>1769079525</v>
+      </c>
+      <c r="B3732" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3732" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3732" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3732" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3732" t="s">
+        <v>3201</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add descriptive statistics for variables (min, max, mean, std)
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -338,6 +338,81 @@
   </si>
   <si>
     <t>13</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__commune</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>12.8</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__annee</t>
+  </si>
+  <si>
+    <t>2005</t>
+  </si>
+  <si>
+    <t>2015.3</t>
+  </si>
+  <si>
+    <t>5.7</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__nb_employes</t>
+  </si>
+  <si>
+    <t>450</t>
+  </si>
+  <si>
+    <t>24.7</t>
+  </si>
+  <si>
+    <t>38.2</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__satisfaction_usagers</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>0.32</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__source_financement</t>
+  </si>
+  <si>
+    <t>-202223</t>
+  </si>
+  <si>
+    <t>4535435</t>
+  </si>
+  <si>
+    <t>2343</t>
+  </si>
+  <si>
+    <t>34.432</t>
   </si>
 </sst>
 </file>
@@ -1559,6 +1634,406 @@
         <v>107</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59">
+        <v>1774122070</v>
+      </c>
+      <c r="B59" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" t="s">
+        <v>5</v>
+      </c>
+      <c r="D59" t="s">
+        <v>108</v>
+      </c>
+      <c r="F59" t="s">
+        <v>109</v>
+      </c>
+      <c r="G59" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>1774122070</v>
+      </c>
+      <c r="B60" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>108</v>
+      </c>
+      <c r="F60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G60" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>1774122070</v>
+      </c>
+      <c r="B61" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>108</v>
+      </c>
+      <c r="F61" t="s">
+        <v>112</v>
+      </c>
+      <c r="G61" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>1774122070</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" t="s">
+        <v>108</v>
+      </c>
+      <c r="F62" t="s">
+        <v>114</v>
+      </c>
+      <c r="G62" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>1774122070</v>
+      </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" t="s">
+        <v>5</v>
+      </c>
+      <c r="D63" t="s">
+        <v>116</v>
+      </c>
+      <c r="F63" t="s">
+        <v>109</v>
+      </c>
+      <c r="G63" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>1774122070</v>
+      </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" t="s">
+        <v>110</v>
+      </c>
+      <c r="G64" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>1774122070</v>
+      </c>
+      <c r="B65" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>116</v>
+      </c>
+      <c r="F65" t="s">
+        <v>112</v>
+      </c>
+      <c r="G65" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>1774122070</v>
+      </c>
+      <c r="B66" t="s">
+        <v>9</v>
+      </c>
+      <c r="C66" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" t="s">
+        <v>116</v>
+      </c>
+      <c r="F66" t="s">
+        <v>114</v>
+      </c>
+      <c r="G66" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>1774122070</v>
+      </c>
+      <c r="B67" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67" t="s">
+        <v>120</v>
+      </c>
+      <c r="F67" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>1774122070</v>
+      </c>
+      <c r="B68" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" t="s">
+        <v>120</v>
+      </c>
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>1774122070</v>
+      </c>
+      <c r="B69" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" t="s">
+        <v>5</v>
+      </c>
+      <c r="D69" t="s">
+        <v>120</v>
+      </c>
+      <c r="F69" t="s">
+        <v>112</v>
+      </c>
+      <c r="G69" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>1774122070</v>
+      </c>
+      <c r="B70" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>120</v>
+      </c>
+      <c r="F70" t="s">
+        <v>114</v>
+      </c>
+      <c r="G70" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>1774122070</v>
+      </c>
+      <c r="B71" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" t="s">
+        <v>124</v>
+      </c>
+      <c r="F71" t="s">
+        <v>109</v>
+      </c>
+      <c r="H71" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>1774122070</v>
+      </c>
+      <c r="B72" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>124</v>
+      </c>
+      <c r="F72" t="s">
+        <v>110</v>
+      </c>
+      <c r="H72" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>1774122070</v>
+      </c>
+      <c r="B73" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" t="s">
+        <v>124</v>
+      </c>
+      <c r="F73" t="s">
+        <v>112</v>
+      </c>
+      <c r="H73" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>1774122070</v>
+      </c>
+      <c r="B74" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" t="s">
+        <v>5</v>
+      </c>
+      <c r="D74" t="s">
+        <v>124</v>
+      </c>
+      <c r="F74" t="s">
+        <v>114</v>
+      </c>
+      <c r="H74" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>1774122070</v>
+      </c>
+      <c r="B75" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" t="s">
+        <v>128</v>
+      </c>
+      <c r="F75" t="s">
+        <v>109</v>
+      </c>
+      <c r="H75" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>1774122070</v>
+      </c>
+      <c r="B76" t="s">
+        <v>9</v>
+      </c>
+      <c r="C76" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" t="s">
+        <v>128</v>
+      </c>
+      <c r="F76" t="s">
+        <v>110</v>
+      </c>
+      <c r="H76" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>1774122070</v>
+      </c>
+      <c r="B77" t="s">
+        <v>9</v>
+      </c>
+      <c r="C77" t="s">
+        <v>5</v>
+      </c>
+      <c r="D77" t="s">
+        <v>128</v>
+      </c>
+      <c r="F77" t="s">
+        <v>112</v>
+      </c>
+      <c r="H77" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>1774122070</v>
+      </c>
+      <c r="B78" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" t="s">
+        <v>5</v>
+      </c>
+      <c r="D78" t="s">
+        <v>128</v>
+      </c>
+      <c r="F78" t="s">
+        <v>114</v>
+      </c>
+      <c r="H78" t="s">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add descriptive statistics for variables (min, max, mean, std) (#95)
* feat: add descriptive statistics for variables (min, max, mean, std)

* docs: clarify instructions regarding modification of build output in app/

* fix: correct baseUrl extraction in getMetaSchema function

* docs: add schema fix to changelog

* release: 0.18.0
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -338,6 +338,81 @@
   </si>
   <si>
     <t>13</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__commune</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>12.8</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__annee</t>
+  </si>
+  <si>
+    <t>2005</t>
+  </si>
+  <si>
+    <t>2015.3</t>
+  </si>
+  <si>
+    <t>5.7</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__nb_employes</t>
+  </si>
+  <si>
+    <t>450</t>
+  </si>
+  <si>
+    <t>24.7</t>
+  </si>
+  <si>
+    <t>38.2</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__satisfaction_usagers</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>0.32</t>
+  </si>
+  <si>
+    <t>ser_pub_loc__source_financement</t>
+  </si>
+  <si>
+    <t>-202223</t>
+  </si>
+  <si>
+    <t>4535435</t>
+  </si>
+  <si>
+    <t>2343</t>
+  </si>
+  <si>
+    <t>34.432</t>
   </si>
 </sst>
 </file>
@@ -1559,6 +1634,406 @@
         <v>107</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59">
+        <v>1774122070</v>
+      </c>
+      <c r="B59" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" t="s">
+        <v>5</v>
+      </c>
+      <c r="D59" t="s">
+        <v>108</v>
+      </c>
+      <c r="F59" t="s">
+        <v>109</v>
+      </c>
+      <c r="G59" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>1774122070</v>
+      </c>
+      <c r="B60" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>108</v>
+      </c>
+      <c r="F60" t="s">
+        <v>110</v>
+      </c>
+      <c r="G60" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>1774122070</v>
+      </c>
+      <c r="B61" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>108</v>
+      </c>
+      <c r="F61" t="s">
+        <v>112</v>
+      </c>
+      <c r="G61" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>1774122070</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" t="s">
+        <v>108</v>
+      </c>
+      <c r="F62" t="s">
+        <v>114</v>
+      </c>
+      <c r="G62" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>1774122070</v>
+      </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" t="s">
+        <v>5</v>
+      </c>
+      <c r="D63" t="s">
+        <v>116</v>
+      </c>
+      <c r="F63" t="s">
+        <v>109</v>
+      </c>
+      <c r="G63" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>1774122070</v>
+      </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" t="s">
+        <v>110</v>
+      </c>
+      <c r="G64" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>1774122070</v>
+      </c>
+      <c r="B65" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>116</v>
+      </c>
+      <c r="F65" t="s">
+        <v>112</v>
+      </c>
+      <c r="G65" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>1774122070</v>
+      </c>
+      <c r="B66" t="s">
+        <v>9</v>
+      </c>
+      <c r="C66" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" t="s">
+        <v>116</v>
+      </c>
+      <c r="F66" t="s">
+        <v>114</v>
+      </c>
+      <c r="G66" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>1774122070</v>
+      </c>
+      <c r="B67" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67" t="s">
+        <v>120</v>
+      </c>
+      <c r="F67" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>1774122070</v>
+      </c>
+      <c r="B68" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" t="s">
+        <v>120</v>
+      </c>
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>1774122070</v>
+      </c>
+      <c r="B69" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" t="s">
+        <v>5</v>
+      </c>
+      <c r="D69" t="s">
+        <v>120</v>
+      </c>
+      <c r="F69" t="s">
+        <v>112</v>
+      </c>
+      <c r="G69" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>1774122070</v>
+      </c>
+      <c r="B70" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>120</v>
+      </c>
+      <c r="F70" t="s">
+        <v>114</v>
+      </c>
+      <c r="G70" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>1774122070</v>
+      </c>
+      <c r="B71" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" t="s">
+        <v>124</v>
+      </c>
+      <c r="F71" t="s">
+        <v>109</v>
+      </c>
+      <c r="H71" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>1774122070</v>
+      </c>
+      <c r="B72" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>124</v>
+      </c>
+      <c r="F72" t="s">
+        <v>110</v>
+      </c>
+      <c r="H72" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>1774122070</v>
+      </c>
+      <c r="B73" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" t="s">
+        <v>124</v>
+      </c>
+      <c r="F73" t="s">
+        <v>112</v>
+      </c>
+      <c r="H73" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>1774122070</v>
+      </c>
+      <c r="B74" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" t="s">
+        <v>5</v>
+      </c>
+      <c r="D74" t="s">
+        <v>124</v>
+      </c>
+      <c r="F74" t="s">
+        <v>114</v>
+      </c>
+      <c r="H74" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>1774122070</v>
+      </c>
+      <c r="B75" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" t="s">
+        <v>128</v>
+      </c>
+      <c r="F75" t="s">
+        <v>109</v>
+      </c>
+      <c r="H75" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>1774122070</v>
+      </c>
+      <c r="B76" t="s">
+        <v>9</v>
+      </c>
+      <c r="C76" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" t="s">
+        <v>128</v>
+      </c>
+      <c r="F76" t="s">
+        <v>110</v>
+      </c>
+      <c r="H76" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>1774122070</v>
+      </c>
+      <c r="B77" t="s">
+        <v>9</v>
+      </c>
+      <c r="C77" t="s">
+        <v>5</v>
+      </c>
+      <c r="D77" t="s">
+        <v>128</v>
+      </c>
+      <c r="F77" t="s">
+        <v>112</v>
+      </c>
+      <c r="H77" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>1774122070</v>
+      </c>
+      <c r="B78" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" t="s">
+        <v>5</v>
+      </c>
+      <c r="D78" t="s">
+        <v>128</v>
+      </c>
+      <c r="F78" t="s">
+        <v>114</v>
+      </c>
+      <c r="H78" t="s">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
improve stats display: date formatting, car. suffix, safeHtml
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -413,6 +413,21 @@
   </si>
   <si>
     <t>34.432</t>
+  </si>
+  <si>
+    <t>pollution_air__date</t>
+  </si>
+  <si>
+    <t>1590102632</t>
+  </si>
+  <si>
+    <t>1774134632</t>
+  </si>
+  <si>
+    <t>1726960232</t>
+  </si>
+  <si>
+    <t>53</t>
   </si>
 </sst>
 </file>
@@ -2034,6 +2049,86 @@
         <v>132</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79">
+        <v>1774134738</v>
+      </c>
+      <c r="B79" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" t="s">
+        <v>5</v>
+      </c>
+      <c r="D79" t="s">
+        <v>133</v>
+      </c>
+      <c r="F79" t="s">
+        <v>109</v>
+      </c>
+      <c r="H79" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>1774134738</v>
+      </c>
+      <c r="B80" t="s">
+        <v>9</v>
+      </c>
+      <c r="C80" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" t="s">
+        <v>133</v>
+      </c>
+      <c r="F80" t="s">
+        <v>110</v>
+      </c>
+      <c r="H80" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>1774134738</v>
+      </c>
+      <c r="B81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" t="s">
+        <v>5</v>
+      </c>
+      <c r="D81" t="s">
+        <v>133</v>
+      </c>
+      <c r="F81" t="s">
+        <v>112</v>
+      </c>
+      <c r="H81" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>1774134738</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" t="s">
+        <v>133</v>
+      </c>
+      <c r="F82" t="s">
+        <v>114</v>
+      </c>
+      <c r="H82" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
improve stats display: date formatting, car. suffix, safeHtml (#97)
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -413,6 +413,21 @@
   </si>
   <si>
     <t>34.432</t>
+  </si>
+  <si>
+    <t>pollution_air__date</t>
+  </si>
+  <si>
+    <t>1590102632</t>
+  </si>
+  <si>
+    <t>1774134632</t>
+  </si>
+  <si>
+    <t>1726960232</t>
+  </si>
+  <si>
+    <t>53</t>
   </si>
 </sst>
 </file>
@@ -2034,6 +2049,86 @@
         <v>132</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79">
+        <v>1774134738</v>
+      </c>
+      <c r="B79" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" t="s">
+        <v>5</v>
+      </c>
+      <c r="D79" t="s">
+        <v>133</v>
+      </c>
+      <c r="F79" t="s">
+        <v>109</v>
+      </c>
+      <c r="H79" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>1774134738</v>
+      </c>
+      <c r="B80" t="s">
+        <v>9</v>
+      </c>
+      <c r="C80" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" t="s">
+        <v>133</v>
+      </c>
+      <c r="F80" t="s">
+        <v>110</v>
+      </c>
+      <c r="H80" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>1774134738</v>
+      </c>
+      <c r="B81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" t="s">
+        <v>5</v>
+      </c>
+      <c r="D81" t="s">
+        <v>133</v>
+      </c>
+      <c r="F81" t="s">
+        <v>112</v>
+      </c>
+      <c r="H81" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>1774134738</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" t="s">
+        <v>133</v>
+      </c>
+      <c r="F82" t="s">
+        <v>114</v>
+      </c>
+      <c r="H82" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: fix variable type column visible even when all variables have no type, now uses raw type for empty column detection
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -455,6 +455,24 @@
   </si>
   <si>
     <t>pop_region</t>
+  </si>
+  <si>
+    <t>tourisme_annu__classification_officielle</t>
+  </si>
+  <si>
+    <t>conso_energie__sous_secteur</t>
+  </si>
+  <si>
+    <t>transport_pub__localite</t>
+  </si>
+  <si>
+    <t>transport_pub__nb_lignes</t>
+  </si>
+  <si>
+    <t>transport_pub__frequence_moyenne</t>
+  </si>
+  <si>
+    <t>float</t>
   </si>
 </sst>
 </file>
@@ -2302,6 +2320,109 @@
         <v>145</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90">
+        <v>1775154977</v>
+      </c>
+      <c r="B90" t="s">
+        <v>9</v>
+      </c>
+      <c r="C90" t="s">
+        <v>5</v>
+      </c>
+      <c r="D90" t="s">
+        <v>147</v>
+      </c>
+      <c r="F90" t="s">
+        <v>1</v>
+      </c>
+      <c r="G90" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>1775154977</v>
+      </c>
+      <c r="B91" t="s">
+        <v>9</v>
+      </c>
+      <c r="C91" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" t="s">
+        <v>148</v>
+      </c>
+      <c r="F91" t="s">
+        <v>1</v>
+      </c>
+      <c r="G91" t="s">
+        <v>11</v>
+      </c>
+      <c r="H91" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>1775155912</v>
+      </c>
+      <c r="B92" t="s">
+        <v>9</v>
+      </c>
+      <c r="C92" t="s">
+        <v>5</v>
+      </c>
+      <c r="D92" t="s">
+        <v>149</v>
+      </c>
+      <c r="F92" t="s">
+        <v>1</v>
+      </c>
+      <c r="G92" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>1775155912</v>
+      </c>
+      <c r="B93" t="s">
+        <v>9</v>
+      </c>
+      <c r="C93" t="s">
+        <v>5</v>
+      </c>
+      <c r="D93" t="s">
+        <v>150</v>
+      </c>
+      <c r="F93" t="s">
+        <v>1</v>
+      </c>
+      <c r="G93" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>1775155912</v>
+      </c>
+      <c r="B94" t="s">
+        <v>9</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" t="s">
+        <v>151</v>
+      </c>
+      <c r="F94" t="s">
+        <v>1</v>
+      </c>
+      <c r="G94" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: fix variable type column visible even when all variables have no type, now uses raw type for empty column detection (#112)
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -455,6 +455,24 @@
   </si>
   <si>
     <t>pop_region</t>
+  </si>
+  <si>
+    <t>tourisme_annu__classification_officielle</t>
+  </si>
+  <si>
+    <t>conso_energie__sous_secteur</t>
+  </si>
+  <si>
+    <t>transport_pub__localite</t>
+  </si>
+  <si>
+    <t>transport_pub__nb_lignes</t>
+  </si>
+  <si>
+    <t>transport_pub__frequence_moyenne</t>
+  </si>
+  <si>
+    <t>float</t>
   </si>
 </sst>
 </file>
@@ -2302,6 +2320,109 @@
         <v>145</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90">
+        <v>1775154977</v>
+      </c>
+      <c r="B90" t="s">
+        <v>9</v>
+      </c>
+      <c r="C90" t="s">
+        <v>5</v>
+      </c>
+      <c r="D90" t="s">
+        <v>147</v>
+      </c>
+      <c r="F90" t="s">
+        <v>1</v>
+      </c>
+      <c r="G90" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>1775154977</v>
+      </c>
+      <c r="B91" t="s">
+        <v>9</v>
+      </c>
+      <c r="C91" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" t="s">
+        <v>148</v>
+      </c>
+      <c r="F91" t="s">
+        <v>1</v>
+      </c>
+      <c r="G91" t="s">
+        <v>11</v>
+      </c>
+      <c r="H91" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>1775155912</v>
+      </c>
+      <c r="B92" t="s">
+        <v>9</v>
+      </c>
+      <c r="C92" t="s">
+        <v>5</v>
+      </c>
+      <c r="D92" t="s">
+        <v>149</v>
+      </c>
+      <c r="F92" t="s">
+        <v>1</v>
+      </c>
+      <c r="G92" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>1775155912</v>
+      </c>
+      <c r="B93" t="s">
+        <v>9</v>
+      </c>
+      <c r="C93" t="s">
+        <v>5</v>
+      </c>
+      <c r="D93" t="s">
+        <v>150</v>
+      </c>
+      <c r="F93" t="s">
+        <v>1</v>
+      </c>
+      <c r="G93" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>1775155912</v>
+      </c>
+      <c r="B94" t="s">
+        <v>9</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" t="s">
+        <v>151</v>
+      </c>
+      <c r="F94" t="s">
+        <v>1</v>
+      </c>
+      <c r="G94" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add: is_pattern attribute for variables with distinct display in freq tab and preview fix: frequency value text overflow and number alignment on multi-line values
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -473,6 +473,75 @@
   </si>
   <si>
     <t>float</t>
+  </si>
+  <si>
+    <t>freq</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite</t>
+  </si>
+  <si>
+    <t>aaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaa-aaaaaa</t>
+  </si>
+  <si>
+    <t>aaa-aaaaaa</t>
+  </si>
+  <si>
+    <t>is_pattern</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaa-aaaaaa-999999999-9999999999-999999999</t>
+  </si>
+  <si>
+    <t>aaa-aaaaaa-999999999-9999999999-999999999</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa9999999999999999999</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa9999999999999999999</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa9999999999999999999aaaaaaaaaaa9999999999aaaaa9999</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa9999999999999999999aaaaaaaaaaa9999999999aaaaa9999</t>
+  </si>
+  <si>
+    <t>canton_sigle---AI</t>
+  </si>
+  <si>
+    <t>Appenzell Rhodes-Intérieures</t>
+  </si>
+  <si>
+    <t>Appenzell Rhodes-Intérieures et autres régions d'ici et d'ailleur et de partout</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>canton_sigle---SZ</t>
+  </si>
+  <si>
+    <t>Schwytz</t>
+  </si>
+  <si>
+    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici</t>
+  </si>
+  <si>
+    <t>SZ</t>
   </si>
 </sst>
 </file>
@@ -2423,6 +2492,253 @@
         <v>152</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95">
+        <v>1776453328</v>
+      </c>
+      <c r="B95" t="s">
+        <v>67</v>
+      </c>
+      <c r="C95" t="s">
+        <v>153</v>
+      </c>
+      <c r="D95" t="s">
+        <v>154</v>
+      </c>
+      <c r="E95" t="s">
+        <v>155</v>
+      </c>
+      <c r="I95" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>1776453328</v>
+      </c>
+      <c r="B96" t="s">
+        <v>67</v>
+      </c>
+      <c r="C96" t="s">
+        <v>153</v>
+      </c>
+      <c r="D96" t="s">
+        <v>157</v>
+      </c>
+      <c r="E96" t="s">
+        <v>155</v>
+      </c>
+      <c r="I96" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>1776453328</v>
+      </c>
+      <c r="B97" t="s">
+        <v>67</v>
+      </c>
+      <c r="C97" t="s">
+        <v>153</v>
+      </c>
+      <c r="D97" t="s">
+        <v>159</v>
+      </c>
+      <c r="E97" t="s">
+        <v>155</v>
+      </c>
+      <c r="I97" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>1776453328</v>
+      </c>
+      <c r="B98" t="s">
+        <v>9</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" t="s">
+        <v>155</v>
+      </c>
+      <c r="F98" t="s">
+        <v>161</v>
+      </c>
+      <c r="H98" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>1776455385</v>
+      </c>
+      <c r="B99" t="s">
+        <v>67</v>
+      </c>
+      <c r="C99" t="s">
+        <v>153</v>
+      </c>
+      <c r="D99" t="s">
+        <v>162</v>
+      </c>
+      <c r="E99" t="s">
+        <v>155</v>
+      </c>
+      <c r="I99" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>1776455422</v>
+      </c>
+      <c r="B100" t="s">
+        <v>67</v>
+      </c>
+      <c r="C100" t="s">
+        <v>153</v>
+      </c>
+      <c r="D100" t="s">
+        <v>164</v>
+      </c>
+      <c r="E100" t="s">
+        <v>155</v>
+      </c>
+      <c r="I100" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>1776455498</v>
+      </c>
+      <c r="B101" t="s">
+        <v>67</v>
+      </c>
+      <c r="C101" t="s">
+        <v>153</v>
+      </c>
+      <c r="D101" t="s">
+        <v>166</v>
+      </c>
+      <c r="E101" t="s">
+        <v>155</v>
+      </c>
+      <c r="I101" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>1776455498</v>
+      </c>
+      <c r="B102" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" t="s">
+        <v>153</v>
+      </c>
+      <c r="D102" t="s">
+        <v>164</v>
+      </c>
+      <c r="E102" t="s">
+        <v>155</v>
+      </c>
+      <c r="I102" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>1776457006</v>
+      </c>
+      <c r="B103" t="s">
+        <v>9</v>
+      </c>
+      <c r="C103" t="s">
+        <v>71</v>
+      </c>
+      <c r="D103" t="s">
+        <v>168</v>
+      </c>
+      <c r="E103" t="s">
+        <v>52</v>
+      </c>
+      <c r="F103" t="s">
+        <v>40</v>
+      </c>
+      <c r="G103" t="s">
+        <v>169</v>
+      </c>
+      <c r="H103" t="s">
+        <v>170</v>
+      </c>
+      <c r="I103" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>1776457062</v>
+      </c>
+      <c r="B104" t="s">
+        <v>9</v>
+      </c>
+      <c r="C104" t="s">
+        <v>71</v>
+      </c>
+      <c r="D104" t="s">
+        <v>172</v>
+      </c>
+      <c r="E104" t="s">
+        <v>52</v>
+      </c>
+      <c r="F104" t="s">
+        <v>40</v>
+      </c>
+      <c r="G104" t="s">
+        <v>173</v>
+      </c>
+      <c r="H104" t="s">
+        <v>174</v>
+      </c>
+      <c r="I104" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>1776457062</v>
+      </c>
+      <c r="B105" t="s">
+        <v>9</v>
+      </c>
+      <c r="C105" t="s">
+        <v>71</v>
+      </c>
+      <c r="D105" t="s">
+        <v>168</v>
+      </c>
+      <c r="E105" t="s">
+        <v>52</v>
+      </c>
+      <c r="F105" t="s">
+        <v>40</v>
+      </c>
+      <c r="G105" t="s">
+        <v>170</v>
+      </c>
+      <c r="H105" t="s">
+        <v>169</v>
+      </c>
+      <c r="I105" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: share button in all modes with link manifest and is_pattern variable attribute (#117)
* add: is_pattern attribute for variables with distinct display in freq tab and preview
fix: frequency value text overflow and number alignment on multi-line values

* feat: share button in all modes with link.json.js manifest

* fix: update dompurify to 3.4.0 and follow-redirects to fix security vulnerabilities
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -473,6 +473,75 @@
   </si>
   <si>
     <t>float</t>
+  </si>
+  <si>
+    <t>freq</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite</t>
+  </si>
+  <si>
+    <t>aaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaa-aaaaaa</t>
+  </si>
+  <si>
+    <t>aaa-aaaaaa</t>
+  </si>
+  <si>
+    <t>is_pattern</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaa-aaaaaa-999999999-9999999999-999999999</t>
+  </si>
+  <si>
+    <t>aaa-aaaaaa-999999999-9999999999-999999999</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa9999999999999999999</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa9999999999999999999</t>
+  </si>
+  <si>
+    <t>emploi_jeunes__nationalite---aaaaaaaaa9999999999999999999aaaaaaaaaaa9999999999aaaaa9999</t>
+  </si>
+  <si>
+    <t>aaaaaaaaa9999999999999999999aaaaaaaaaaa9999999999aaaaa9999</t>
+  </si>
+  <si>
+    <t>canton_sigle---AI</t>
+  </si>
+  <si>
+    <t>Appenzell Rhodes-Intérieures</t>
+  </si>
+  <si>
+    <t>Appenzell Rhodes-Intérieures et autres régions d'ici et d'ailleur et de partout</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>canton_sigle---SZ</t>
+  </si>
+  <si>
+    <t>Schwytz</t>
+  </si>
+  <si>
+    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici</t>
+  </si>
+  <si>
+    <t>SZ</t>
   </si>
 </sst>
 </file>
@@ -2423,6 +2492,253 @@
         <v>152</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95">
+        <v>1776453328</v>
+      </c>
+      <c r="B95" t="s">
+        <v>67</v>
+      </c>
+      <c r="C95" t="s">
+        <v>153</v>
+      </c>
+      <c r="D95" t="s">
+        <v>154</v>
+      </c>
+      <c r="E95" t="s">
+        <v>155</v>
+      </c>
+      <c r="I95" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>1776453328</v>
+      </c>
+      <c r="B96" t="s">
+        <v>67</v>
+      </c>
+      <c r="C96" t="s">
+        <v>153</v>
+      </c>
+      <c r="D96" t="s">
+        <v>157</v>
+      </c>
+      <c r="E96" t="s">
+        <v>155</v>
+      </c>
+      <c r="I96" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>1776453328</v>
+      </c>
+      <c r="B97" t="s">
+        <v>67</v>
+      </c>
+      <c r="C97" t="s">
+        <v>153</v>
+      </c>
+      <c r="D97" t="s">
+        <v>159</v>
+      </c>
+      <c r="E97" t="s">
+        <v>155</v>
+      </c>
+      <c r="I97" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>1776453328</v>
+      </c>
+      <c r="B98" t="s">
+        <v>9</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" t="s">
+        <v>155</v>
+      </c>
+      <c r="F98" t="s">
+        <v>161</v>
+      </c>
+      <c r="H98" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>1776455385</v>
+      </c>
+      <c r="B99" t="s">
+        <v>67</v>
+      </c>
+      <c r="C99" t="s">
+        <v>153</v>
+      </c>
+      <c r="D99" t="s">
+        <v>162</v>
+      </c>
+      <c r="E99" t="s">
+        <v>155</v>
+      </c>
+      <c r="I99" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>1776455422</v>
+      </c>
+      <c r="B100" t="s">
+        <v>67</v>
+      </c>
+      <c r="C100" t="s">
+        <v>153</v>
+      </c>
+      <c r="D100" t="s">
+        <v>164</v>
+      </c>
+      <c r="E100" t="s">
+        <v>155</v>
+      </c>
+      <c r="I100" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>1776455498</v>
+      </c>
+      <c r="B101" t="s">
+        <v>67</v>
+      </c>
+      <c r="C101" t="s">
+        <v>153</v>
+      </c>
+      <c r="D101" t="s">
+        <v>166</v>
+      </c>
+      <c r="E101" t="s">
+        <v>155</v>
+      </c>
+      <c r="I101" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>1776455498</v>
+      </c>
+      <c r="B102" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" t="s">
+        <v>153</v>
+      </c>
+      <c r="D102" t="s">
+        <v>164</v>
+      </c>
+      <c r="E102" t="s">
+        <v>155</v>
+      </c>
+      <c r="I102" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>1776457006</v>
+      </c>
+      <c r="B103" t="s">
+        <v>9</v>
+      </c>
+      <c r="C103" t="s">
+        <v>71</v>
+      </c>
+      <c r="D103" t="s">
+        <v>168</v>
+      </c>
+      <c r="E103" t="s">
+        <v>52</v>
+      </c>
+      <c r="F103" t="s">
+        <v>40</v>
+      </c>
+      <c r="G103" t="s">
+        <v>169</v>
+      </c>
+      <c r="H103" t="s">
+        <v>170</v>
+      </c>
+      <c r="I103" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>1776457062</v>
+      </c>
+      <c r="B104" t="s">
+        <v>9</v>
+      </c>
+      <c r="C104" t="s">
+        <v>71</v>
+      </c>
+      <c r="D104" t="s">
+        <v>172</v>
+      </c>
+      <c r="E104" t="s">
+        <v>52</v>
+      </c>
+      <c r="F104" t="s">
+        <v>40</v>
+      </c>
+      <c r="G104" t="s">
+        <v>173</v>
+      </c>
+      <c r="H104" t="s">
+        <v>174</v>
+      </c>
+      <c r="I104" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>1776457062</v>
+      </c>
+      <c r="B105" t="s">
+        <v>9</v>
+      </c>
+      <c r="C105" t="s">
+        <v>71</v>
+      </c>
+      <c r="D105" t="s">
+        <v>168</v>
+      </c>
+      <c r="E105" t="s">
+        <v>52</v>
+      </c>
+      <c r="F105" t="s">
+        <v>40</v>
+      </c>
+      <c r="G105" t="s">
+        <v>170</v>
+      </c>
+      <c r="H105" t="s">
+        <v>169</v>
+      </c>
+      <c r="I105" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add concept glossary entity
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF04864B-DB8C-7347-95F2-D2FEBD49D7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="176">
   <si>
     <t>timestamp</t>
   </si>
@@ -547,18 +553,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <color theme="1"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <b/>
-      <color theme="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -578,17 +586,350 @@
       <diagonal/>
     </border>
   </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
   <cellXfs count="2">
-    <xf/>
-    <xf fontId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I105"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1737208669</v>
       </c>
@@ -640,7 +981,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1737633510</v>
       </c>
@@ -663,7 +1004,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1737633510</v>
       </c>
@@ -686,7 +1027,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1737635096</v>
       </c>
@@ -709,7 +1050,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1737638842</v>
       </c>
@@ -732,7 +1073,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1737638842</v>
       </c>
@@ -755,7 +1096,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1737639740</v>
       </c>
@@ -778,7 +1119,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1746359037</v>
       </c>
@@ -801,7 +1142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1746734601</v>
       </c>
@@ -821,7 +1162,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1746734601</v>
       </c>
@@ -841,7 +1182,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1746734601</v>
       </c>
@@ -861,7 +1202,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1747315104</v>
       </c>
@@ -884,7 +1225,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1747315150</v>
       </c>
@@ -904,7 +1245,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1747315514</v>
       </c>
@@ -924,7 +1265,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1747315514</v>
       </c>
@@ -944,7 +1285,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1747315529</v>
       </c>
@@ -964,7 +1305,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1747315547</v>
       </c>
@@ -984,7 +1325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1747315547</v>
       </c>
@@ -1004,7 +1345,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1747315547</v>
       </c>
@@ -1024,7 +1365,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1747315547</v>
       </c>
@@ -1044,7 +1385,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1747315547</v>
       </c>
@@ -1064,7 +1405,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1747340787</v>
       </c>
@@ -1084,7 +1425,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1747340787</v>
       </c>
@@ -1104,7 +1445,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1747340787</v>
       </c>
@@ -1124,7 +1465,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1747340787</v>
       </c>
@@ -1144,7 +1485,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1747906147</v>
       </c>
@@ -1164,7 +1505,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1747906281</v>
       </c>
@@ -1178,7 +1519,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1747906551</v>
       </c>
@@ -1198,7 +1539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1747906551</v>
       </c>
@@ -1218,7 +1559,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1747906566</v>
       </c>
@@ -1241,7 +1582,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1747907576</v>
       </c>
@@ -1255,7 +1596,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>1747907576</v>
       </c>
@@ -1269,7 +1610,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1747907625</v>
       </c>
@@ -1283,7 +1624,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1747907625</v>
       </c>
@@ -1297,7 +1638,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>1747913177</v>
       </c>
@@ -1311,7 +1652,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>1747913221</v>
       </c>
@@ -1331,7 +1672,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>1747913221</v>
       </c>
@@ -1351,7 +1692,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>1747913314</v>
       </c>
@@ -1371,7 +1712,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1747913314</v>
       </c>
@@ -1391,7 +1732,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1747918633</v>
       </c>
@@ -1411,7 +1752,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1747921769</v>
       </c>
@@ -1431,7 +1772,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1747921769</v>
       </c>
@@ -1451,7 +1792,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1747921769</v>
       </c>
@@ -1471,7 +1812,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1749897806</v>
       </c>
@@ -1485,7 +1826,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>1749897806</v>
       </c>
@@ -1499,7 +1840,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1759431975</v>
       </c>
@@ -1522,7 +1863,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>1759432050</v>
       </c>
@@ -1545,7 +1886,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1759435301</v>
       </c>
@@ -1574,7 +1915,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1759435408</v>
       </c>
@@ -1594,7 +1935,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>1759435408</v>
       </c>
@@ -1614,7 +1955,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1759443360</v>
       </c>
@@ -1634,7 +1975,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>1759443360</v>
       </c>
@@ -1654,7 +1995,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>1759778989</v>
       </c>
@@ -1677,7 +2018,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>1760952632</v>
       </c>
@@ -1700,7 +2041,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>1774082203</v>
       </c>
@@ -1720,7 +2061,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>1774082203</v>
       </c>
@@ -1740,7 +2081,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>1774084450</v>
       </c>
@@ -1763,7 +2104,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>1774122070</v>
       </c>
@@ -1783,7 +2124,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>1774122070</v>
       </c>
@@ -1803,7 +2144,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>1774122070</v>
       </c>
@@ -1823,7 +2164,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>1774122070</v>
       </c>
@@ -1843,7 +2184,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>1774122070</v>
       </c>
@@ -1863,7 +2204,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>1774122070</v>
       </c>
@@ -1883,7 +2224,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>1774122070</v>
       </c>
@@ -1903,7 +2244,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>1774122070</v>
       </c>
@@ -1923,7 +2264,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>1774122070</v>
       </c>
@@ -1943,7 +2284,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>1774122070</v>
       </c>
@@ -1963,7 +2304,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>1774122070</v>
       </c>
@@ -1983,7 +2324,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>1774122070</v>
       </c>
@@ -2003,7 +2344,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>1774122070</v>
       </c>
@@ -2023,7 +2364,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>1774122070</v>
       </c>
@@ -2043,7 +2384,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>1774122070</v>
       </c>
@@ -2063,7 +2404,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>1774122070</v>
       </c>
@@ -2083,7 +2424,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>1774122070</v>
       </c>
@@ -2103,7 +2444,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>1774122070</v>
       </c>
@@ -2123,7 +2464,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>1774122070</v>
       </c>
@@ -2143,7 +2484,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>1774122070</v>
       </c>
@@ -2163,7 +2504,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>1774134738</v>
       </c>
@@ -2183,7 +2524,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>1774134738</v>
       </c>
@@ -2203,7 +2544,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>1774134738</v>
       </c>
@@ -2223,7 +2564,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>1774134738</v>
       </c>
@@ -2243,7 +2584,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>1774985291</v>
       </c>
@@ -2266,7 +2607,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>1774987898</v>
       </c>
@@ -2289,7 +2630,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>1775142369</v>
       </c>
@@ -2309,7 +2650,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>1775143200</v>
       </c>
@@ -2329,7 +2670,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>1775143200</v>
       </c>
@@ -2349,7 +2690,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>1775143256</v>
       </c>
@@ -2369,7 +2710,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>1775143273</v>
       </c>
@@ -2389,7 +2730,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>1775154977</v>
       </c>
@@ -2409,7 +2750,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>1775154977</v>
       </c>
@@ -2432,7 +2773,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>1775155912</v>
       </c>
@@ -2452,7 +2793,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>1775155912</v>
       </c>
@@ -2472,7 +2813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>1775155912</v>
       </c>
@@ -2492,7 +2833,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>1776453328</v>
       </c>
@@ -2512,7 +2853,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>1776453328</v>
       </c>
@@ -2532,7 +2873,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>1776453328</v>
       </c>
@@ -2552,7 +2893,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>1776453328</v>
       </c>
@@ -2572,7 +2913,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>1776455385</v>
       </c>
@@ -2592,7 +2933,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>1776455422</v>
       </c>
@@ -2612,7 +2953,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>1776455498</v>
       </c>
@@ -2632,7 +2973,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>1776455498</v>
       </c>
@@ -2652,7 +2993,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>1776457006</v>
       </c>
@@ -2681,7 +3022,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>1776457062</v>
       </c>
@@ -2710,7 +3051,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>1776457062</v>
       </c>
@@ -2740,5 +3081,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add concept glossary entity (#119)
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF04864B-DB8C-7347-95F2-D2FEBD49D7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="176">
   <si>
     <t>timestamp</t>
   </si>
@@ -547,18 +553,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <color theme="1"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <b/>
-      <color theme="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -578,17 +586,350 @@
       <diagonal/>
     </border>
   </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
   <cellXfs count="2">
-    <xf/>
-    <xf fontId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I105"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1737208669</v>
       </c>
@@ -640,7 +981,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1737633510</v>
       </c>
@@ -663,7 +1004,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1737633510</v>
       </c>
@@ -686,7 +1027,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1737635096</v>
       </c>
@@ -709,7 +1050,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1737638842</v>
       </c>
@@ -732,7 +1073,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1737638842</v>
       </c>
@@ -755,7 +1096,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1737639740</v>
       </c>
@@ -778,7 +1119,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1746359037</v>
       </c>
@@ -801,7 +1142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1746734601</v>
       </c>
@@ -821,7 +1162,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1746734601</v>
       </c>
@@ -841,7 +1182,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1746734601</v>
       </c>
@@ -861,7 +1202,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1747315104</v>
       </c>
@@ -884,7 +1225,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1747315150</v>
       </c>
@@ -904,7 +1245,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1747315514</v>
       </c>
@@ -924,7 +1265,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1747315514</v>
       </c>
@@ -944,7 +1285,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1747315529</v>
       </c>
@@ -964,7 +1305,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1747315547</v>
       </c>
@@ -984,7 +1325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1747315547</v>
       </c>
@@ -1004,7 +1345,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1747315547</v>
       </c>
@@ -1024,7 +1365,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1747315547</v>
       </c>
@@ -1044,7 +1385,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1747315547</v>
       </c>
@@ -1064,7 +1405,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1747340787</v>
       </c>
@@ -1084,7 +1425,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1747340787</v>
       </c>
@@ -1104,7 +1445,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1747340787</v>
       </c>
@@ -1124,7 +1465,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1747340787</v>
       </c>
@@ -1144,7 +1485,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1747906147</v>
       </c>
@@ -1164,7 +1505,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1747906281</v>
       </c>
@@ -1178,7 +1519,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1747906551</v>
       </c>
@@ -1198,7 +1539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1747906551</v>
       </c>
@@ -1218,7 +1559,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1747906566</v>
       </c>
@@ -1241,7 +1582,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1747907576</v>
       </c>
@@ -1255,7 +1596,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>1747907576</v>
       </c>
@@ -1269,7 +1610,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1747907625</v>
       </c>
@@ -1283,7 +1624,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1747907625</v>
       </c>
@@ -1297,7 +1638,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>1747913177</v>
       </c>
@@ -1311,7 +1652,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>1747913221</v>
       </c>
@@ -1331,7 +1672,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>1747913221</v>
       </c>
@@ -1351,7 +1692,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>1747913314</v>
       </c>
@@ -1371,7 +1712,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1747913314</v>
       </c>
@@ -1391,7 +1732,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1747918633</v>
       </c>
@@ -1411,7 +1752,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1747921769</v>
       </c>
@@ -1431,7 +1772,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1747921769</v>
       </c>
@@ -1451,7 +1792,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1747921769</v>
       </c>
@@ -1471,7 +1812,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1749897806</v>
       </c>
@@ -1485,7 +1826,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>1749897806</v>
       </c>
@@ -1499,7 +1840,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1759431975</v>
       </c>
@@ -1522,7 +1863,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>1759432050</v>
       </c>
@@ -1545,7 +1886,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1759435301</v>
       </c>
@@ -1574,7 +1915,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1759435408</v>
       </c>
@@ -1594,7 +1935,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>1759435408</v>
       </c>
@@ -1614,7 +1955,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1759443360</v>
       </c>
@@ -1634,7 +1975,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>1759443360</v>
       </c>
@@ -1654,7 +1995,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>1759778989</v>
       </c>
@@ -1677,7 +2018,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>1760952632</v>
       </c>
@@ -1700,7 +2041,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>1774082203</v>
       </c>
@@ -1720,7 +2061,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>1774082203</v>
       </c>
@@ -1740,7 +2081,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>1774084450</v>
       </c>
@@ -1763,7 +2104,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>1774122070</v>
       </c>
@@ -1783,7 +2124,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>1774122070</v>
       </c>
@@ -1803,7 +2144,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>1774122070</v>
       </c>
@@ -1823,7 +2164,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>1774122070</v>
       </c>
@@ -1843,7 +2184,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>1774122070</v>
       </c>
@@ -1863,7 +2204,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>1774122070</v>
       </c>
@@ -1883,7 +2224,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>1774122070</v>
       </c>
@@ -1903,7 +2244,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>1774122070</v>
       </c>
@@ -1923,7 +2264,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>1774122070</v>
       </c>
@@ -1943,7 +2284,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>1774122070</v>
       </c>
@@ -1963,7 +2304,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>1774122070</v>
       </c>
@@ -1983,7 +2324,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>1774122070</v>
       </c>
@@ -2003,7 +2344,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>1774122070</v>
       </c>
@@ -2023,7 +2364,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>1774122070</v>
       </c>
@@ -2043,7 +2384,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>1774122070</v>
       </c>
@@ -2063,7 +2404,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>1774122070</v>
       </c>
@@ -2083,7 +2424,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>1774122070</v>
       </c>
@@ -2103,7 +2444,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>1774122070</v>
       </c>
@@ -2123,7 +2464,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>1774122070</v>
       </c>
@@ -2143,7 +2484,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>1774122070</v>
       </c>
@@ -2163,7 +2504,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>1774134738</v>
       </c>
@@ -2183,7 +2524,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>1774134738</v>
       </c>
@@ -2203,7 +2544,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>1774134738</v>
       </c>
@@ -2223,7 +2564,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>1774134738</v>
       </c>
@@ -2243,7 +2584,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>1774985291</v>
       </c>
@@ -2266,7 +2607,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>1774987898</v>
       </c>
@@ -2289,7 +2630,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>1775142369</v>
       </c>
@@ -2309,7 +2650,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>1775143200</v>
       </c>
@@ -2329,7 +2670,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>1775143200</v>
       </c>
@@ -2349,7 +2690,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>1775143256</v>
       </c>
@@ -2369,7 +2710,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>1775143273</v>
       </c>
@@ -2389,7 +2730,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>1775154977</v>
       </c>
@@ -2409,7 +2750,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>1775154977</v>
       </c>
@@ -2432,7 +2773,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>1775155912</v>
       </c>
@@ -2452,7 +2793,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>1775155912</v>
       </c>
@@ -2472,7 +2813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>1775155912</v>
       </c>
@@ -2492,7 +2833,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>1776453328</v>
       </c>
@@ -2512,7 +2853,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>1776453328</v>
       </c>
@@ -2532,7 +2873,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>1776453328</v>
       </c>
@@ -2552,7 +2893,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>1776453328</v>
       </c>
@@ -2572,7 +2913,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>1776455385</v>
       </c>
@@ -2592,7 +2933,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>1776455422</v>
       </c>
@@ -2612,7 +2953,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>1776455498</v>
       </c>
@@ -2632,7 +2973,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>1776455498</v>
       </c>
@@ -2652,7 +2993,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>1776457006</v>
       </c>
@@ -2681,7 +3022,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>1776457062</v>
       </c>
@@ -2710,7 +3051,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>1776457062</v>
       </c>
@@ -2740,5 +3081,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rename institution entity to organization
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF04864B-DB8C-7347-95F2-D2FEBD49D7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DB771D-3464-374B-A220-8C9BA69BBD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -190,9 +190,6 @@
     <t>vide</t>
   </si>
   <si>
-    <t>institution</t>
-  </si>
-  <si>
     <t>dfi</t>
   </si>
   <si>
@@ -548,6 +545,9 @@
   </si>
   <si>
     <t>SZ</t>
+  </si>
+  <si>
+    <t>organization</t>
   </si>
 </sst>
 </file>
@@ -1413,16 +1413,16 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
+        <v>175</v>
+      </c>
+      <c r="D23" t="s">
         <v>56</v>
-      </c>
-      <c r="D23" t="s">
-        <v>57</v>
       </c>
       <c r="F23" t="s">
         <v>15</v>
       </c>
       <c r="H23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -1433,16 +1433,16 @@
         <v>9</v>
       </c>
       <c r="C24" t="s">
+        <v>175</v>
+      </c>
+      <c r="D24" t="s">
         <v>56</v>
-      </c>
-      <c r="D24" t="s">
-        <v>57</v>
       </c>
       <c r="F24" t="s">
         <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -1453,16 +1453,16 @@
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>175</v>
       </c>
       <c r="D25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F25" t="s">
         <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -1473,16 +1473,16 @@
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
+        <v>175</v>
       </c>
       <c r="D26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F26" t="s">
         <v>18</v>
       </c>
       <c r="H26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -1496,13 +1496,13 @@
         <v>5</v>
       </c>
       <c r="D27" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27" t="s">
         <v>64</v>
       </c>
-      <c r="F27" t="s">
+      <c r="H27" t="s">
         <v>65</v>
-      </c>
-      <c r="H27" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -1510,13 +1510,13 @@
         <v>1747906281</v>
       </c>
       <c r="B28" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>68</v>
-      </c>
-      <c r="D28" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -1530,13 +1530,13 @@
         <v>5</v>
       </c>
       <c r="D29" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" t="s">
         <v>64</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>65</v>
-      </c>
-      <c r="G29" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -1550,13 +1550,13 @@
         <v>5</v>
       </c>
       <c r="D30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -1567,19 +1567,19 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" t="s">
         <v>68</v>
       </c>
-      <c r="D31" t="s">
-        <v>69</v>
-      </c>
       <c r="F31" t="s">
+        <v>70</v>
+      </c>
+      <c r="G31" t="s">
         <v>71</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>72</v>
-      </c>
-      <c r="H31" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -1587,13 +1587,13 @@
         <v>1747907576</v>
       </c>
       <c r="B32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" t="s">
         <v>67</v>
       </c>
-      <c r="C32" t="s">
-        <v>68</v>
-      </c>
       <c r="D32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -1604,10 +1604,10 @@
         <v>43</v>
       </c>
       <c r="C33" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" t="s">
         <v>68</v>
-      </c>
-      <c r="D33" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -1615,13 +1615,13 @@
         <v>1747907625</v>
       </c>
       <c r="B34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" t="s">
         <v>67</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>68</v>
-      </c>
-      <c r="D34" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -1632,10 +1632,10 @@
         <v>43</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -1646,10 +1646,10 @@
         <v>43</v>
       </c>
       <c r="C36" t="s">
+        <v>67</v>
+      </c>
+      <c r="D36" t="s">
         <v>68</v>
-      </c>
-      <c r="D36" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -1663,13 +1663,13 @@
         <v>5</v>
       </c>
       <c r="D37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -1683,13 +1683,13 @@
         <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -1703,13 +1703,13 @@
         <v>5</v>
       </c>
       <c r="D39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -1723,13 +1723,13 @@
         <v>5</v>
       </c>
       <c r="D40" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -1743,13 +1743,13 @@
         <v>5</v>
       </c>
       <c r="D41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H41" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -1763,13 +1763,13 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" t="s">
+        <v>69</v>
+      </c>
+      <c r="H42" t="s">
         <v>77</v>
-      </c>
-      <c r="F42" t="s">
-        <v>70</v>
-      </c>
-      <c r="H42" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -1783,13 +1783,13 @@
         <v>5</v>
       </c>
       <c r="D43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -1806,10 +1806,10 @@
         <v>33</v>
       </c>
       <c r="F44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H44" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -1817,13 +1817,13 @@
         <v>1749897806</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C45" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" t="s">
         <v>81</v>
-      </c>
-      <c r="D45" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -1831,13 +1831,13 @@
         <v>1749897806</v>
       </c>
       <c r="B46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D46" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -1848,16 +1848,16 @@
         <v>9</v>
       </c>
       <c r="C47" t="s">
+        <v>83</v>
+      </c>
+      <c r="D47" t="s">
         <v>84</v>
-      </c>
-      <c r="D47" t="s">
-        <v>85</v>
       </c>
       <c r="F47" t="s">
         <v>18</v>
       </c>
       <c r="G47" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H47" t="s">
         <v>19</v>
@@ -1871,19 +1871,19 @@
         <v>9</v>
       </c>
       <c r="C48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F48" t="s">
         <v>40</v>
       </c>
       <c r="G48" t="s">
+        <v>86</v>
+      </c>
+      <c r="H48" t="s">
         <v>87</v>
-      </c>
-      <c r="H48" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
@@ -1894,10 +1894,10 @@
         <v>9</v>
       </c>
       <c r="C49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E49" t="s">
         <v>53</v>
@@ -1906,13 +1906,13 @@
         <v>40</v>
       </c>
       <c r="G49" t="s">
+        <v>87</v>
+      </c>
+      <c r="H49" t="s">
         <v>88</v>
       </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>89</v>
-      </c>
-      <c r="I49" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
@@ -1920,19 +1920,19 @@
         <v>1759435408</v>
       </c>
       <c r="B50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E50" t="s">
         <v>49</v>
       </c>
       <c r="I50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
@@ -1943,16 +1943,16 @@
         <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E51" t="s">
         <v>49</v>
       </c>
       <c r="I51" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
@@ -1960,19 +1960,19 @@
         <v>1759443360</v>
       </c>
       <c r="B52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D52" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E52" t="s">
         <v>49</v>
       </c>
       <c r="I52" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
@@ -1983,16 +1983,16 @@
         <v>43</v>
       </c>
       <c r="C53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E53" t="s">
         <v>49</v>
       </c>
       <c r="I53" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
@@ -2003,19 +2003,19 @@
         <v>9</v>
       </c>
       <c r="C54" t="s">
+        <v>94</v>
+      </c>
+      <c r="D54" t="s">
         <v>95</v>
       </c>
-      <c r="D54" t="s">
+      <c r="F54" t="s">
         <v>96</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>97</v>
       </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>98</v>
-      </c>
-      <c r="H54" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
@@ -2026,19 +2026,19 @@
         <v>9</v>
       </c>
       <c r="C55" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F55" t="s">
         <v>40</v>
       </c>
       <c r="G55" t="s">
+        <v>100</v>
+      </c>
+      <c r="H55" t="s">
         <v>101</v>
-      </c>
-      <c r="H55" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
@@ -2052,13 +2052,13 @@
         <v>13</v>
       </c>
       <c r="D56" t="s">
+        <v>102</v>
+      </c>
+      <c r="F56" t="s">
         <v>103</v>
       </c>
-      <c r="F56" t="s">
+      <c r="H56" t="s">
         <v>104</v>
-      </c>
-      <c r="H56" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
@@ -2075,10 +2075,10 @@
         <v>30</v>
       </c>
       <c r="F57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H57" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
@@ -2095,13 +2095,13 @@
         <v>30</v>
       </c>
       <c r="F58" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G58" t="s">
+        <v>105</v>
+      </c>
+      <c r="H58" t="s">
         <v>106</v>
-      </c>
-      <c r="H58" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
@@ -2115,13 +2115,13 @@
         <v>5</v>
       </c>
       <c r="D59" t="s">
+        <v>107</v>
+      </c>
+      <c r="F59" t="s">
         <v>108</v>
       </c>
-      <c r="F59" t="s">
-        <v>109</v>
-      </c>
       <c r="G59" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
@@ -2135,13 +2135,13 @@
         <v>5</v>
       </c>
       <c r="D60" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F60" t="s">
+        <v>109</v>
+      </c>
+      <c r="G60" t="s">
         <v>110</v>
-      </c>
-      <c r="G60" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
@@ -2155,13 +2155,13 @@
         <v>5</v>
       </c>
       <c r="D61" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F61" t="s">
+        <v>111</v>
+      </c>
+      <c r="G61" t="s">
         <v>112</v>
-      </c>
-      <c r="G61" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
@@ -2175,13 +2175,13 @@
         <v>5</v>
       </c>
       <c r="D62" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F62" t="s">
+        <v>113</v>
+      </c>
+      <c r="G62" t="s">
         <v>114</v>
-      </c>
-      <c r="G62" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
@@ -2195,13 +2195,13 @@
         <v>5</v>
       </c>
       <c r="D63" t="s">
+        <v>115</v>
+      </c>
+      <c r="F63" t="s">
+        <v>108</v>
+      </c>
+      <c r="G63" t="s">
         <v>116</v>
-      </c>
-      <c r="F63" t="s">
-        <v>109</v>
-      </c>
-      <c r="G63" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
@@ -2215,10 +2215,10 @@
         <v>5</v>
       </c>
       <c r="D64" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F64" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G64" t="s">
         <v>19</v>
@@ -2235,13 +2235,13 @@
         <v>5</v>
       </c>
       <c r="D65" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F65" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G65" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -2255,13 +2255,13 @@
         <v>5</v>
       </c>
       <c r="D66" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F66" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G66" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -2275,10 +2275,10 @@
         <v>5</v>
       </c>
       <c r="D67" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F67" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G67" t="s">
         <v>36</v>
@@ -2295,13 +2295,13 @@
         <v>5</v>
       </c>
       <c r="D68" t="s">
+        <v>119</v>
+      </c>
+      <c r="F68" t="s">
+        <v>109</v>
+      </c>
+      <c r="G68" t="s">
         <v>120</v>
-      </c>
-      <c r="F68" t="s">
-        <v>110</v>
-      </c>
-      <c r="G68" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -2315,13 +2315,13 @@
         <v>5</v>
       </c>
       <c r="D69" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F69" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G69" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -2335,13 +2335,13 @@
         <v>5</v>
       </c>
       <c r="D70" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G70" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
@@ -2355,13 +2355,13 @@
         <v>5</v>
       </c>
       <c r="D71" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F71" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H71" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -2375,13 +2375,13 @@
         <v>5</v>
       </c>
       <c r="D72" t="s">
+        <v>123</v>
+      </c>
+      <c r="F72" t="s">
+        <v>109</v>
+      </c>
+      <c r="H72" t="s">
         <v>124</v>
-      </c>
-      <c r="F72" t="s">
-        <v>110</v>
-      </c>
-      <c r="H72" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -2395,13 +2395,13 @@
         <v>5</v>
       </c>
       <c r="D73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
@@ -2415,13 +2415,13 @@
         <v>5</v>
       </c>
       <c r="D74" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F74" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H74" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
@@ -2435,13 +2435,13 @@
         <v>5</v>
       </c>
       <c r="D75" t="s">
+        <v>127</v>
+      </c>
+      <c r="F75" t="s">
+        <v>108</v>
+      </c>
+      <c r="H75" t="s">
         <v>128</v>
-      </c>
-      <c r="F75" t="s">
-        <v>109</v>
-      </c>
-      <c r="H75" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
@@ -2455,13 +2455,13 @@
         <v>5</v>
       </c>
       <c r="D76" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F76" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H76" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
@@ -2475,13 +2475,13 @@
         <v>5</v>
       </c>
       <c r="D77" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F77" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H77" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
@@ -2495,13 +2495,13 @@
         <v>5</v>
       </c>
       <c r="D78" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H78" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
@@ -2515,13 +2515,13 @@
         <v>5</v>
       </c>
       <c r="D79" t="s">
+        <v>132</v>
+      </c>
+      <c r="F79" t="s">
+        <v>108</v>
+      </c>
+      <c r="H79" t="s">
         <v>133</v>
-      </c>
-      <c r="F79" t="s">
-        <v>109</v>
-      </c>
-      <c r="H79" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
@@ -2535,13 +2535,13 @@
         <v>5</v>
       </c>
       <c r="D80" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F80" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H80" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
@@ -2555,13 +2555,13 @@
         <v>5</v>
       </c>
       <c r="D81" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F81" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H81" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
@@ -2575,13 +2575,13 @@
         <v>5</v>
       </c>
       <c r="D82" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F82" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H82" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
@@ -2595,7 +2595,7 @@
         <v>5</v>
       </c>
       <c r="D83" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F83" t="s">
         <v>1</v>
@@ -2604,7 +2604,7 @@
         <v>11</v>
       </c>
       <c r="H83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
@@ -2621,13 +2621,13 @@
         <v>30</v>
       </c>
       <c r="F84" t="s">
+        <v>139</v>
+      </c>
+      <c r="G84" t="s">
         <v>140</v>
       </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
         <v>141</v>
-      </c>
-      <c r="H84" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
@@ -2641,13 +2641,13 @@
         <v>13</v>
       </c>
       <c r="D85" t="s">
+        <v>142</v>
+      </c>
+      <c r="F85" t="s">
         <v>143</v>
       </c>
-      <c r="F85" t="s">
+      <c r="H85" t="s">
         <v>144</v>
-      </c>
-      <c r="H85" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
@@ -2661,13 +2661,13 @@
         <v>13</v>
       </c>
       <c r="D86" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F86" t="s">
+        <v>143</v>
+      </c>
+      <c r="H86" t="s">
         <v>144</v>
-      </c>
-      <c r="H86" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
@@ -2681,13 +2681,13 @@
         <v>13</v>
       </c>
       <c r="D87" t="s">
+        <v>142</v>
+      </c>
+      <c r="F87" t="s">
         <v>143</v>
       </c>
-      <c r="F87" t="s">
+      <c r="G87" t="s">
         <v>144</v>
-      </c>
-      <c r="G87" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
@@ -2701,13 +2701,13 @@
         <v>13</v>
       </c>
       <c r="D88" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F88" t="s">
+        <v>143</v>
+      </c>
+      <c r="G88" t="s">
         <v>144</v>
-      </c>
-      <c r="G88" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
@@ -2721,13 +2721,13 @@
         <v>13</v>
       </c>
       <c r="D89" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F89" t="s">
+        <v>143</v>
+      </c>
+      <c r="H89" t="s">
         <v>144</v>
-      </c>
-      <c r="H89" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
@@ -2741,7 +2741,7 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F90" t="s">
         <v>1</v>
@@ -2761,7 +2761,7 @@
         <v>5</v>
       </c>
       <c r="D91" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F91" t="s">
         <v>1</v>
@@ -2770,7 +2770,7 @@
         <v>11</v>
       </c>
       <c r="H91" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
@@ -2784,7 +2784,7 @@
         <v>5</v>
       </c>
       <c r="D92" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F92" t="s">
         <v>1</v>
@@ -2804,7 +2804,7 @@
         <v>5</v>
       </c>
       <c r="D93" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F93" t="s">
         <v>1</v>
@@ -2824,13 +2824,13 @@
         <v>5</v>
       </c>
       <c r="D94" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F94" t="s">
         <v>1</v>
       </c>
       <c r="G94" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
@@ -2838,19 +2838,19 @@
         <v>1776453328</v>
       </c>
       <c r="B95" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C95" t="s">
+        <v>152</v>
+      </c>
+      <c r="D95" t="s">
         <v>153</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E95" t="s">
         <v>154</v>
       </c>
-      <c r="E95" t="s">
+      <c r="I95" t="s">
         <v>155</v>
-      </c>
-      <c r="I95" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
@@ -2858,19 +2858,19 @@
         <v>1776453328</v>
       </c>
       <c r="B96" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C96" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D96" t="s">
+        <v>156</v>
+      </c>
+      <c r="E96" t="s">
+        <v>154</v>
+      </c>
+      <c r="I96" t="s">
         <v>157</v>
-      </c>
-      <c r="E96" t="s">
-        <v>155</v>
-      </c>
-      <c r="I96" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
@@ -2878,19 +2878,19 @@
         <v>1776453328</v>
       </c>
       <c r="B97" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C97" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D97" t="s">
+        <v>158</v>
+      </c>
+      <c r="E97" t="s">
+        <v>154</v>
+      </c>
+      <c r="I97" t="s">
         <v>159</v>
-      </c>
-      <c r="E97" t="s">
-        <v>155</v>
-      </c>
-      <c r="I97" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
@@ -2904,10 +2904,10 @@
         <v>5</v>
       </c>
       <c r="D98" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F98" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H98" t="s">
         <v>36</v>
@@ -2918,19 +2918,19 @@
         <v>1776455385</v>
       </c>
       <c r="B99" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C99" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D99" t="s">
+        <v>161</v>
+      </c>
+      <c r="E99" t="s">
+        <v>154</v>
+      </c>
+      <c r="I99" t="s">
         <v>162</v>
-      </c>
-      <c r="E99" t="s">
-        <v>155</v>
-      </c>
-      <c r="I99" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.2">
@@ -2938,19 +2938,19 @@
         <v>1776455422</v>
       </c>
       <c r="B100" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C100" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D100" t="s">
+        <v>163</v>
+      </c>
+      <c r="E100" t="s">
+        <v>154</v>
+      </c>
+      <c r="I100" t="s">
         <v>164</v>
-      </c>
-      <c r="E100" t="s">
-        <v>155</v>
-      </c>
-      <c r="I100" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
@@ -2958,19 +2958,19 @@
         <v>1776455498</v>
       </c>
       <c r="B101" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C101" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D101" t="s">
+        <v>165</v>
+      </c>
+      <c r="E101" t="s">
+        <v>154</v>
+      </c>
+      <c r="I101" t="s">
         <v>166</v>
-      </c>
-      <c r="E101" t="s">
-        <v>155</v>
-      </c>
-      <c r="I101" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
@@ -2981,16 +2981,16 @@
         <v>43</v>
       </c>
       <c r="C102" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D102" t="s">
+        <v>163</v>
+      </c>
+      <c r="E102" t="s">
+        <v>154</v>
+      </c>
+      <c r="I102" t="s">
         <v>164</v>
-      </c>
-      <c r="E102" t="s">
-        <v>155</v>
-      </c>
-      <c r="I102" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
@@ -3001,10 +3001,10 @@
         <v>9</v>
       </c>
       <c r="C103" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D103" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E103" t="s">
         <v>52</v>
@@ -3013,13 +3013,13 @@
         <v>40</v>
       </c>
       <c r="G103" t="s">
+        <v>168</v>
+      </c>
+      <c r="H103" t="s">
         <v>169</v>
       </c>
-      <c r="H103" t="s">
+      <c r="I103" t="s">
         <v>170</v>
-      </c>
-      <c r="I103" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
@@ -3030,10 +3030,10 @@
         <v>9</v>
       </c>
       <c r="C104" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D104" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E104" t="s">
         <v>52</v>
@@ -3042,13 +3042,13 @@
         <v>40</v>
       </c>
       <c r="G104" t="s">
+        <v>172</v>
+      </c>
+      <c r="H104" t="s">
         <v>173</v>
       </c>
-      <c r="H104" t="s">
+      <c r="I104" t="s">
         <v>174</v>
-      </c>
-      <c r="I104" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
@@ -3059,10 +3059,10 @@
         <v>9</v>
       </c>
       <c r="C105" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D105" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E105" t="s">
         <v>52</v>
@@ -3071,13 +3071,13 @@
         <v>40</v>
       </c>
       <c r="G105" t="s">
+        <v>169</v>
+      </c>
+      <c r="H105" t="s">
+        <v>168</v>
+      </c>
+      <c r="I105" t="s">
         <v>170</v>
-      </c>
-      <c r="H105" t="s">
-        <v>169</v>
-      </c>
-      <c r="I105" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update evolution for frequency rename
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DB771D-3464-374B-A220-8C9BA69BBD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>timestamp</t>
   </si>
@@ -190,6 +184,9 @@
     <t>vide</t>
   </si>
   <si>
+    <t>organization</t>
+  </si>
+  <si>
     <t>dfi</t>
   </si>
   <si>
@@ -478,7 +475,7 @@
     <t>float</t>
   </si>
   <si>
-    <t>freq</t>
+    <t>frequency</t>
   </si>
   <si>
     <t>emploi_jeunes__nationalite---aaaaaa</t>
@@ -547,26 +544,177 @@
     <t>SZ</t>
   </si>
   <si>
-    <t>organization</t>
+    <t>pop_region__population_totale---value</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>frequencyuency</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_1</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>value_1</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_2</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>value_2</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_3</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>value_3</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_4</t>
+  </si>
+  <si>
+    <t>value_4</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_5</t>
+  </si>
+  <si>
+    <t>value_5</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_6</t>
+  </si>
+  <si>
+    <t>value_6</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_7</t>
+  </si>
+  <si>
+    <t>value_7</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_8</t>
+  </si>
+  <si>
+    <t>value_8</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_9</t>
+  </si>
+  <si>
+    <t>value_9</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_10</t>
+  </si>
+  <si>
+    <t>value_10</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_11</t>
+  </si>
+  <si>
+    <t>value_11</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_12</t>
+  </si>
+  <si>
+    <t>value_12</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_13</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>value_13</t>
+  </si>
+  <si>
+    <t>pop_region__population_totale---value_14</t>
+  </si>
+  <si>
+    <t>value_14</t>
+  </si>
+  <si>
+    <t>pop_region__type_region---urbaine</t>
+  </si>
+  <si>
+    <t>pop_region__type_region</t>
+  </si>
+  <si>
+    <t>9432</t>
+  </si>
+  <si>
+    <t>urbaine</t>
+  </si>
+  <si>
+    <t>pop_region__type_region---priurbaine</t>
+  </si>
+  <si>
+    <t>périurbaine</t>
+  </si>
+  <si>
+    <t>pop_region__type_region---rurale</t>
+  </si>
+  <si>
+    <t>3434</t>
+  </si>
+  <si>
+    <t>rurale</t>
+  </si>
+  <si>
+    <t>pop_region__type_region---montagne</t>
+  </si>
+  <si>
+    <t>9481</t>
+  </si>
+  <si>
+    <t>montagne</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>46</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
-      <sz val="12"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <scheme val="minor"/>
       <b/>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -586,350 +734,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf/>
+    <xf fontId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I105"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +773,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2">
         <v>1737208669</v>
       </c>
@@ -981,7 +796,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3">
         <v>1737633510</v>
       </c>
@@ -1004,7 +819,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4">
         <v>1737633510</v>
       </c>
@@ -1027,7 +842,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5">
         <v>1737635096</v>
       </c>
@@ -1050,7 +865,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6">
         <v>1737638842</v>
       </c>
@@ -1073,7 +888,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7">
         <v>1737638842</v>
       </c>
@@ -1096,7 +911,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8">
         <v>1737639740</v>
       </c>
@@ -1119,7 +934,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9">
         <v>1746359037</v>
       </c>
@@ -1142,7 +957,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10">
         <v>1746734601</v>
       </c>
@@ -1162,7 +977,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11">
         <v>1746734601</v>
       </c>
@@ -1182,7 +997,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12">
         <v>1746734601</v>
       </c>
@@ -1202,7 +1017,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13">
         <v>1747315104</v>
       </c>
@@ -1225,7 +1040,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14">
         <v>1747315150</v>
       </c>
@@ -1245,7 +1060,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15">
       <c r="A15">
         <v>1747315514</v>
       </c>
@@ -1265,7 +1080,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16">
         <v>1747315514</v>
       </c>
@@ -1285,7 +1100,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17">
         <v>1747315529</v>
       </c>
@@ -1305,7 +1120,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18">
       <c r="A18">
         <v>1747315547</v>
       </c>
@@ -1325,7 +1140,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19">
         <v>1747315547</v>
       </c>
@@ -1345,7 +1160,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20">
       <c r="A20">
         <v>1747315547</v>
       </c>
@@ -1365,7 +1180,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21">
         <v>1747315547</v>
       </c>
@@ -1385,7 +1200,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22">
         <v>1747315547</v>
       </c>
@@ -1405,7 +1220,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23">
         <v>1747340787</v>
       </c>
@@ -1413,19 +1228,19 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
         <v>15</v>
       </c>
       <c r="H23" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24">
         <v>1747340787</v>
       </c>
@@ -1433,19 +1248,19 @@
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F24" t="s">
         <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25">
         <v>1747340787</v>
       </c>
@@ -1453,19 +1268,19 @@
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F25" t="s">
         <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26">
         <v>1747340787</v>
       </c>
@@ -1473,19 +1288,19 @@
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F26" t="s">
         <v>18</v>
       </c>
       <c r="H26" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27">
         <v>1747906147</v>
       </c>
@@ -1496,30 +1311,30 @@
         <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H27" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28">
         <v>1747906281</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29">
         <v>1747906551</v>
       </c>
@@ -1530,16 +1345,16 @@
         <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G29" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30">
         <v>1747906551</v>
       </c>
@@ -1550,16 +1365,16 @@
         <v>5</v>
       </c>
       <c r="D30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H30" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31">
         <v>1747906566</v>
       </c>
@@ -1567,36 +1382,36 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H31" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32">
         <v>1747907576</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D32" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33">
         <v>1747907576</v>
       </c>
@@ -1604,27 +1419,27 @@
         <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34">
         <v>1747907625</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35">
         <v>1747907625</v>
       </c>
@@ -1632,13 +1447,13 @@
         <v>43</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36">
         <v>1747913177</v>
       </c>
@@ -1646,13 +1461,13 @@
         <v>43</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37">
       <c r="A37">
         <v>1747913221</v>
       </c>
@@ -1663,16 +1478,16 @@
         <v>5</v>
       </c>
       <c r="D37" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G37" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38">
         <v>1747913221</v>
       </c>
@@ -1683,16 +1498,16 @@
         <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H38" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39">
         <v>1747913314</v>
       </c>
@@ -1703,16 +1518,16 @@
         <v>5</v>
       </c>
       <c r="D39" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F39" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40">
         <v>1747913314</v>
       </c>
@@ -1723,16 +1538,16 @@
         <v>5</v>
       </c>
       <c r="D40" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F40" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H40" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41">
         <v>1747918633</v>
       </c>
@@ -1743,16 +1558,16 @@
         <v>5</v>
       </c>
       <c r="D41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F41" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H41" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42">
         <v>1747921769</v>
       </c>
@@ -1763,16 +1578,16 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F42" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H42" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43">
         <v>1747921769</v>
       </c>
@@ -1783,16 +1598,16 @@
         <v>5</v>
       </c>
       <c r="D43" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" t="s">
+        <v>70</v>
+      </c>
+      <c r="H43" t="s">
         <v>78</v>
       </c>
-      <c r="F43" t="s">
-        <v>69</v>
-      </c>
-      <c r="H43" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44">
       <c r="A44">
         <v>1747921769</v>
       </c>
@@ -1806,41 +1621,41 @@
         <v>33</v>
       </c>
       <c r="F44" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H44" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45">
         <v>1749897806</v>
       </c>
       <c r="B45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D45" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="46">
       <c r="A46">
         <v>1749897806</v>
       </c>
       <c r="B46" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C46" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D46" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47">
       <c r="A47">
         <v>1759431975</v>
       </c>
@@ -1848,22 +1663,22 @@
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D47" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F47" t="s">
         <v>18</v>
       </c>
       <c r="G47" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H47" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48">
       <c r="A48">
         <v>1759432050</v>
       </c>
@@ -1871,22 +1686,22 @@
         <v>9</v>
       </c>
       <c r="C48" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D48" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F48" t="s">
         <v>40</v>
       </c>
       <c r="G48" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H48" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49">
         <v>1759435301</v>
       </c>
@@ -1894,10 +1709,10 @@
         <v>9</v>
       </c>
       <c r="C49" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D49" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E49" t="s">
         <v>53</v>
@@ -1906,36 +1721,36 @@
         <v>40</v>
       </c>
       <c r="G49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H49" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I49" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="50">
       <c r="A50">
         <v>1759435408</v>
       </c>
       <c r="B50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E50" t="s">
         <v>49</v>
       </c>
       <c r="I50" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51">
         <v>1759435408</v>
       </c>
@@ -1943,39 +1758,39 @@
         <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D51" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E51" t="s">
         <v>49</v>
       </c>
       <c r="I51" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52">
         <v>1759443360</v>
       </c>
       <c r="B52" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C52" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D52" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E52" t="s">
         <v>49</v>
       </c>
       <c r="I52" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53">
         <v>1759443360</v>
       </c>
@@ -1983,19 +1798,19 @@
         <v>43</v>
       </c>
       <c r="C53" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D53" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E53" t="s">
         <v>49</v>
       </c>
       <c r="I53" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54">
         <v>1759778989</v>
       </c>
@@ -2003,22 +1818,22 @@
         <v>9</v>
       </c>
       <c r="C54" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D54" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F54" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G54" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H54" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="55">
       <c r="A55">
         <v>1760952632</v>
       </c>
@@ -2026,22 +1841,22 @@
         <v>9</v>
       </c>
       <c r="C55" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D55" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F55" t="s">
         <v>40</v>
       </c>
       <c r="G55" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H55" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="56">
       <c r="A56">
         <v>1774082203</v>
       </c>
@@ -2052,16 +1867,16 @@
         <v>13</v>
       </c>
       <c r="D56" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F56" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H56" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="57">
       <c r="A57">
         <v>1774082203</v>
       </c>
@@ -2075,13 +1890,13 @@
         <v>30</v>
       </c>
       <c r="F57" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H57" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58">
       <c r="A58">
         <v>1774084450</v>
       </c>
@@ -2095,16 +1910,16 @@
         <v>30</v>
       </c>
       <c r="F58" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G58" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H58" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="59">
       <c r="A59">
         <v>1774122070</v>
       </c>
@@ -2115,16 +1930,16 @@
         <v>5</v>
       </c>
       <c r="D59" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F59" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G59" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60">
       <c r="A60">
         <v>1774122070</v>
       </c>
@@ -2135,16 +1950,16 @@
         <v>5</v>
       </c>
       <c r="D60" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F60" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G60" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61">
       <c r="A61">
         <v>1774122070</v>
       </c>
@@ -2155,16 +1970,16 @@
         <v>5</v>
       </c>
       <c r="D61" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F61" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G61" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="62">
       <c r="A62">
         <v>1774122070</v>
       </c>
@@ -2175,16 +1990,16 @@
         <v>5</v>
       </c>
       <c r="D62" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F62" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G62" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63">
       <c r="A63">
         <v>1774122070</v>
       </c>
@@ -2195,16 +2010,16 @@
         <v>5</v>
       </c>
       <c r="D63" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F63" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G63" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64">
       <c r="A64">
         <v>1774122070</v>
       </c>
@@ -2215,16 +2030,16 @@
         <v>5</v>
       </c>
       <c r="D64" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F64" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G64" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65">
       <c r="A65">
         <v>1774122070</v>
       </c>
@@ -2235,16 +2050,16 @@
         <v>5</v>
       </c>
       <c r="D65" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F65" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G65" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66">
       <c r="A66">
         <v>1774122070</v>
       </c>
@@ -2255,16 +2070,16 @@
         <v>5</v>
       </c>
       <c r="D66" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F66" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G66" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="67">
       <c r="A67">
         <v>1774122070</v>
       </c>
@@ -2275,16 +2090,16 @@
         <v>5</v>
       </c>
       <c r="D67" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F67" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G67" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68">
       <c r="A68">
         <v>1774122070</v>
       </c>
@@ -2295,16 +2110,16 @@
         <v>5</v>
       </c>
       <c r="D68" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F68" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G68" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="69">
       <c r="A69">
         <v>1774122070</v>
       </c>
@@ -2315,16 +2130,16 @@
         <v>5</v>
       </c>
       <c r="D69" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F69" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G69" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70">
       <c r="A70">
         <v>1774122070</v>
       </c>
@@ -2335,16 +2150,16 @@
         <v>5</v>
       </c>
       <c r="D70" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F70" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G70" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71">
       <c r="A71">
         <v>1774122070</v>
       </c>
@@ -2355,16 +2170,16 @@
         <v>5</v>
       </c>
       <c r="D71" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F71" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H71" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72">
       <c r="A72">
         <v>1774122070</v>
       </c>
@@ -2375,16 +2190,16 @@
         <v>5</v>
       </c>
       <c r="D72" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F72" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H72" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73">
       <c r="A73">
         <v>1774122070</v>
       </c>
@@ -2395,16 +2210,16 @@
         <v>5</v>
       </c>
       <c r="D73" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F73" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H73" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74">
       <c r="A74">
         <v>1774122070</v>
       </c>
@@ -2415,16 +2230,16 @@
         <v>5</v>
       </c>
       <c r="D74" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F74" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H74" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75">
       <c r="A75">
         <v>1774122070</v>
       </c>
@@ -2435,16 +2250,16 @@
         <v>5</v>
       </c>
       <c r="D75" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F75" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H75" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="76">
       <c r="A76">
         <v>1774122070</v>
       </c>
@@ -2455,16 +2270,16 @@
         <v>5</v>
       </c>
       <c r="D76" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F76" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H76" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="77">
       <c r="A77">
         <v>1774122070</v>
       </c>
@@ -2475,16 +2290,16 @@
         <v>5</v>
       </c>
       <c r="D77" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F77" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H77" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="78">
       <c r="A78">
         <v>1774122070</v>
       </c>
@@ -2495,16 +2310,16 @@
         <v>5</v>
       </c>
       <c r="D78" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F78" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H78" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="79">
       <c r="A79">
         <v>1774134738</v>
       </c>
@@ -2515,16 +2330,16 @@
         <v>5</v>
       </c>
       <c r="D79" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F79" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H79" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="80">
       <c r="A80">
         <v>1774134738</v>
       </c>
@@ -2535,16 +2350,16 @@
         <v>5</v>
       </c>
       <c r="D80" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F80" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H80" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="81">
       <c r="A81">
         <v>1774134738</v>
       </c>
@@ -2555,16 +2370,16 @@
         <v>5</v>
       </c>
       <c r="D81" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F81" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H81" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="82">
       <c r="A82">
         <v>1774134738</v>
       </c>
@@ -2575,16 +2390,16 @@
         <v>5</v>
       </c>
       <c r="D82" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F82" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H82" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="83">
       <c r="A83">
         <v>1774985291</v>
       </c>
@@ -2595,7 +2410,7 @@
         <v>5</v>
       </c>
       <c r="D83" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F83" t="s">
         <v>1</v>
@@ -2604,10 +2419,10 @@
         <v>11</v>
       </c>
       <c r="H83" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="84">
       <c r="A84">
         <v>1774987898</v>
       </c>
@@ -2621,16 +2436,16 @@
         <v>30</v>
       </c>
       <c r="F84" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G84" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H84" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="85">
       <c r="A85">
         <v>1775142369</v>
       </c>
@@ -2641,16 +2456,16 @@
         <v>13</v>
       </c>
       <c r="D85" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F85" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H85" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="86">
       <c r="A86">
         <v>1775143200</v>
       </c>
@@ -2661,16 +2476,16 @@
         <v>13</v>
       </c>
       <c r="D86" t="s">
+        <v>146</v>
+      </c>
+      <c r="F86" t="s">
+        <v>144</v>
+      </c>
+      <c r="H86" t="s">
         <v>145</v>
       </c>
-      <c r="F86" t="s">
-        <v>143</v>
-      </c>
-      <c r="H86" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="87">
       <c r="A87">
         <v>1775143200</v>
       </c>
@@ -2681,16 +2496,16 @@
         <v>13</v>
       </c>
       <c r="D87" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F87" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G87" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88">
       <c r="A88">
         <v>1775143256</v>
       </c>
@@ -2701,16 +2516,16 @@
         <v>13</v>
       </c>
       <c r="D88" t="s">
+        <v>146</v>
+      </c>
+      <c r="F88" t="s">
+        <v>144</v>
+      </c>
+      <c r="G88" t="s">
         <v>145</v>
       </c>
-      <c r="F88" t="s">
-        <v>143</v>
-      </c>
-      <c r="G88" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="89">
       <c r="A89">
         <v>1775143273</v>
       </c>
@@ -2721,16 +2536,16 @@
         <v>13</v>
       </c>
       <c r="D89" t="s">
+        <v>146</v>
+      </c>
+      <c r="F89" t="s">
+        <v>144</v>
+      </c>
+      <c r="H89" t="s">
         <v>145</v>
       </c>
-      <c r="F89" t="s">
-        <v>143</v>
-      </c>
-      <c r="H89" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="90">
       <c r="A90">
         <v>1775154977</v>
       </c>
@@ -2741,7 +2556,7 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F90" t="s">
         <v>1</v>
@@ -2750,7 +2565,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="91">
       <c r="A91">
         <v>1775154977</v>
       </c>
@@ -2761,7 +2576,7 @@
         <v>5</v>
       </c>
       <c r="D91" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F91" t="s">
         <v>1</v>
@@ -2770,10 +2585,10 @@
         <v>11</v>
       </c>
       <c r="H91" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="92">
       <c r="A92">
         <v>1775155912</v>
       </c>
@@ -2784,7 +2599,7 @@
         <v>5</v>
       </c>
       <c r="D92" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F92" t="s">
         <v>1</v>
@@ -2793,7 +2608,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="93">
       <c r="A93">
         <v>1775155912</v>
       </c>
@@ -2804,7 +2619,7 @@
         <v>5</v>
       </c>
       <c r="D93" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F93" t="s">
         <v>1</v>
@@ -2813,7 +2628,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="94">
       <c r="A94">
         <v>1775155912</v>
       </c>
@@ -2824,76 +2639,76 @@
         <v>5</v>
       </c>
       <c r="D94" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F94" t="s">
         <v>1</v>
       </c>
       <c r="G94" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="95">
       <c r="A95">
         <v>1776453328</v>
       </c>
       <c r="B95" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C95" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D95" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E95" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I95" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="96">
       <c r="A96">
         <v>1776453328</v>
       </c>
       <c r="B96" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C96" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D96" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E96" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I96" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="97">
       <c r="A97">
         <v>1776453328</v>
       </c>
       <c r="B97" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C97" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D97" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E97" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I97" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="98">
       <c r="A98">
         <v>1776453328</v>
       </c>
@@ -2904,76 +2719,76 @@
         <v>5</v>
       </c>
       <c r="D98" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F98" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H98" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="99">
       <c r="A99">
         <v>1776455385</v>
       </c>
       <c r="B99" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C99" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D99" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E99" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I99" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="100">
       <c r="A100">
         <v>1776455422</v>
       </c>
       <c r="B100" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C100" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D100" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E100" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I100" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="101">
       <c r="A101">
         <v>1776455498</v>
       </c>
       <c r="B101" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C101" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D101" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E101" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I101" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="102">
       <c r="A102">
         <v>1776455498</v>
       </c>
@@ -2981,19 +2796,19 @@
         <v>43</v>
       </c>
       <c r="C102" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D102" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E102" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I102" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="103">
       <c r="A103">
         <v>1776457006</v>
       </c>
@@ -3001,10 +2816,10 @@
         <v>9</v>
       </c>
       <c r="C103" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D103" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E103" t="s">
         <v>52</v>
@@ -3013,16 +2828,16 @@
         <v>40</v>
       </c>
       <c r="G103" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H103" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I103" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="104">
       <c r="A104">
         <v>1776457062</v>
       </c>
@@ -3030,10 +2845,10 @@
         <v>9</v>
       </c>
       <c r="C104" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D104" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E104" t="s">
         <v>52</v>
@@ -3042,16 +2857,16 @@
         <v>40</v>
       </c>
       <c r="G104" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H104" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I104" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="105">
       <c r="A105">
         <v>1776457062</v>
       </c>
@@ -3059,10 +2874,10 @@
         <v>9</v>
       </c>
       <c r="C105" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D105" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E105" t="s">
         <v>52</v>
@@ -3071,16 +2886,1292 @@
         <v>40</v>
       </c>
       <c r="G105" t="s">
+        <v>170</v>
+      </c>
+      <c r="H105" t="s">
         <v>169</v>
       </c>
-      <c r="H105" t="s">
-        <v>168</v>
-      </c>
       <c r="I105" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>1777402020</v>
+      </c>
+      <c r="B106" t="s">
+        <v>9</v>
+      </c>
+      <c r="C106" t="s">
+        <v>153</v>
+      </c>
+      <c r="D106" t="s">
+        <v>176</v>
+      </c>
+      <c r="E106" t="s">
+        <v>177</v>
+      </c>
+      <c r="F106" t="s">
+        <v>153</v>
+      </c>
+      <c r="G106" t="s">
+        <v>178</v>
+      </c>
+      <c r="I106" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>1777402020</v>
+      </c>
+      <c r="B107" t="s">
+        <v>9</v>
+      </c>
+      <c r="C107" t="s">
+        <v>153</v>
+      </c>
+      <c r="D107" t="s">
+        <v>176</v>
+      </c>
+      <c r="E107" t="s">
+        <v>177</v>
+      </c>
+      <c r="F107" t="s">
+        <v>179</v>
+      </c>
+      <c r="H107" t="s">
+        <v>178</v>
+      </c>
+      <c r="I107" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>1777402020</v>
+      </c>
+      <c r="B108" t="s">
+        <v>9</v>
+      </c>
+      <c r="C108" t="s">
+        <v>153</v>
+      </c>
+      <c r="D108" t="s">
+        <v>180</v>
+      </c>
+      <c r="E108" t="s">
+        <v>177</v>
+      </c>
+      <c r="F108" t="s">
+        <v>153</v>
+      </c>
+      <c r="G108" t="s">
+        <v>181</v>
+      </c>
+      <c r="I108" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>1777402020</v>
+      </c>
+      <c r="B109" t="s">
+        <v>9</v>
+      </c>
+      <c r="C109" t="s">
+        <v>153</v>
+      </c>
+      <c r="D109" t="s">
+        <v>180</v>
+      </c>
+      <c r="E109" t="s">
+        <v>177</v>
+      </c>
+      <c r="F109" t="s">
+        <v>179</v>
+      </c>
+      <c r="H109" t="s">
+        <v>181</v>
+      </c>
+      <c r="I109" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>1777402020</v>
+      </c>
+      <c r="B110" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110" t="s">
+        <v>153</v>
+      </c>
+      <c r="D110" t="s">
+        <v>183</v>
+      </c>
+      <c r="E110" t="s">
+        <v>177</v>
+      </c>
+      <c r="F110" t="s">
+        <v>153</v>
+      </c>
+      <c r="G110" t="s">
+        <v>184</v>
+      </c>
+      <c r="I110" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>1777402020</v>
+      </c>
+      <c r="B111" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" t="s">
+        <v>153</v>
+      </c>
+      <c r="D111" t="s">
+        <v>183</v>
+      </c>
+      <c r="E111" t="s">
+        <v>177</v>
+      </c>
+      <c r="F111" t="s">
+        <v>179</v>
+      </c>
+      <c r="H111" t="s">
+        <v>184</v>
+      </c>
+      <c r="I111" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>1777402020</v>
+      </c>
+      <c r="B112" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" t="s">
+        <v>153</v>
+      </c>
+      <c r="D112" t="s">
+        <v>186</v>
+      </c>
+      <c r="E112" t="s">
+        <v>177</v>
+      </c>
+      <c r="F112" t="s">
+        <v>153</v>
+      </c>
+      <c r="G112" t="s">
+        <v>187</v>
+      </c>
+      <c r="I112" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>1777402020</v>
+      </c>
+      <c r="B113" t="s">
+        <v>9</v>
+      </c>
+      <c r="C113" t="s">
+        <v>153</v>
+      </c>
+      <c r="D113" t="s">
+        <v>186</v>
+      </c>
+      <c r="E113" t="s">
+        <v>177</v>
+      </c>
+      <c r="F113" t="s">
+        <v>179</v>
+      </c>
+      <c r="H113" t="s">
+        <v>187</v>
+      </c>
+      <c r="I113" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>1777402020</v>
+      </c>
+      <c r="B114" t="s">
+        <v>9</v>
+      </c>
+      <c r="C114" t="s">
+        <v>153</v>
+      </c>
+      <c r="D114" t="s">
+        <v>189</v>
+      </c>
+      <c r="E114" t="s">
+        <v>177</v>
+      </c>
+      <c r="F114" t="s">
+        <v>153</v>
+      </c>
+      <c r="G114" t="s">
+        <v>187</v>
+      </c>
+      <c r="I114" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>1777402020</v>
+      </c>
+      <c r="B115" t="s">
+        <v>9</v>
+      </c>
+      <c r="C115" t="s">
+        <v>153</v>
+      </c>
+      <c r="D115" t="s">
+        <v>189</v>
+      </c>
+      <c r="E115" t="s">
+        <v>177</v>
+      </c>
+      <c r="F115" t="s">
+        <v>179</v>
+      </c>
+      <c r="H115" t="s">
+        <v>187</v>
+      </c>
+      <c r="I115" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>1777402020</v>
+      </c>
+      <c r="B116" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" t="s">
+        <v>153</v>
+      </c>
+      <c r="D116" t="s">
+        <v>191</v>
+      </c>
+      <c r="E116" t="s">
+        <v>177</v>
+      </c>
+      <c r="F116" t="s">
+        <v>153</v>
+      </c>
+      <c r="G116" t="s">
+        <v>187</v>
+      </c>
+      <c r="I116" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>1777402020</v>
+      </c>
+      <c r="B117" t="s">
+        <v>9</v>
+      </c>
+      <c r="C117" t="s">
+        <v>153</v>
+      </c>
+      <c r="D117" t="s">
+        <v>191</v>
+      </c>
+      <c r="E117" t="s">
+        <v>177</v>
+      </c>
+      <c r="F117" t="s">
+        <v>179</v>
+      </c>
+      <c r="H117" t="s">
+        <v>187</v>
+      </c>
+      <c r="I117" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>1777402020</v>
+      </c>
+      <c r="B118" t="s">
+        <v>9</v>
+      </c>
+      <c r="C118" t="s">
+        <v>153</v>
+      </c>
+      <c r="D118" t="s">
+        <v>193</v>
+      </c>
+      <c r="E118" t="s">
+        <v>177</v>
+      </c>
+      <c r="F118" t="s">
+        <v>153</v>
+      </c>
+      <c r="G118" t="s">
+        <v>187</v>
+      </c>
+      <c r="I118" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>1777402020</v>
+      </c>
+      <c r="B119" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119" t="s">
+        <v>153</v>
+      </c>
+      <c r="D119" t="s">
+        <v>193</v>
+      </c>
+      <c r="E119" t="s">
+        <v>177</v>
+      </c>
+      <c r="F119" t="s">
+        <v>179</v>
+      </c>
+      <c r="H119" t="s">
+        <v>187</v>
+      </c>
+      <c r="I119" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>1777402020</v>
+      </c>
+      <c r="B120" t="s">
+        <v>9</v>
+      </c>
+      <c r="C120" t="s">
+        <v>153</v>
+      </c>
+      <c r="D120" t="s">
+        <v>195</v>
+      </c>
+      <c r="E120" t="s">
+        <v>177</v>
+      </c>
+      <c r="F120" t="s">
+        <v>153</v>
+      </c>
+      <c r="G120" t="s">
+        <v>187</v>
+      </c>
+      <c r="I120" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>1777402020</v>
+      </c>
+      <c r="B121" t="s">
+        <v>9</v>
+      </c>
+      <c r="C121" t="s">
+        <v>153</v>
+      </c>
+      <c r="D121" t="s">
+        <v>195</v>
+      </c>
+      <c r="E121" t="s">
+        <v>177</v>
+      </c>
+      <c r="F121" t="s">
+        <v>179</v>
+      </c>
+      <c r="H121" t="s">
+        <v>187</v>
+      </c>
+      <c r="I121" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>1777402020</v>
+      </c>
+      <c r="B122" t="s">
+        <v>9</v>
+      </c>
+      <c r="C122" t="s">
+        <v>153</v>
+      </c>
+      <c r="D122" t="s">
+        <v>197</v>
+      </c>
+      <c r="E122" t="s">
+        <v>177</v>
+      </c>
+      <c r="F122" t="s">
+        <v>153</v>
+      </c>
+      <c r="G122" t="s">
+        <v>187</v>
+      </c>
+      <c r="I122" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>1777402020</v>
+      </c>
+      <c r="B123" t="s">
+        <v>9</v>
+      </c>
+      <c r="C123" t="s">
+        <v>153</v>
+      </c>
+      <c r="D123" t="s">
+        <v>197</v>
+      </c>
+      <c r="E123" t="s">
+        <v>177</v>
+      </c>
+      <c r="F123" t="s">
+        <v>179</v>
+      </c>
+      <c r="H123" t="s">
+        <v>187</v>
+      </c>
+      <c r="I123" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>1777402020</v>
+      </c>
+      <c r="B124" t="s">
+        <v>9</v>
+      </c>
+      <c r="C124" t="s">
+        <v>153</v>
+      </c>
+      <c r="D124" t="s">
+        <v>199</v>
+      </c>
+      <c r="E124" t="s">
+        <v>177</v>
+      </c>
+      <c r="F124" t="s">
+        <v>153</v>
+      </c>
+      <c r="G124" t="s">
+        <v>187</v>
+      </c>
+      <c r="I124" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>1777402020</v>
+      </c>
+      <c r="B125" t="s">
+        <v>9</v>
+      </c>
+      <c r="C125" t="s">
+        <v>153</v>
+      </c>
+      <c r="D125" t="s">
+        <v>199</v>
+      </c>
+      <c r="E125" t="s">
+        <v>177</v>
+      </c>
+      <c r="F125" t="s">
+        <v>179</v>
+      </c>
+      <c r="H125" t="s">
+        <v>187</v>
+      </c>
+      <c r="I125" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>1777402020</v>
+      </c>
+      <c r="B126" t="s">
+        <v>9</v>
+      </c>
+      <c r="C126" t="s">
+        <v>153</v>
+      </c>
+      <c r="D126" t="s">
+        <v>201</v>
+      </c>
+      <c r="E126" t="s">
+        <v>177</v>
+      </c>
+      <c r="F126" t="s">
+        <v>153</v>
+      </c>
+      <c r="G126" t="s">
+        <v>187</v>
+      </c>
+      <c r="I126" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>1777402020</v>
+      </c>
+      <c r="B127" t="s">
+        <v>9</v>
+      </c>
+      <c r="C127" t="s">
+        <v>153</v>
+      </c>
+      <c r="D127" t="s">
+        <v>201</v>
+      </c>
+      <c r="E127" t="s">
+        <v>177</v>
+      </c>
+      <c r="F127" t="s">
+        <v>179</v>
+      </c>
+      <c r="H127" t="s">
+        <v>187</v>
+      </c>
+      <c r="I127" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>1777402020</v>
+      </c>
+      <c r="B128" t="s">
+        <v>9</v>
+      </c>
+      <c r="C128" t="s">
+        <v>153</v>
+      </c>
+      <c r="D128" t="s">
+        <v>203</v>
+      </c>
+      <c r="E128" t="s">
+        <v>177</v>
+      </c>
+      <c r="F128" t="s">
+        <v>153</v>
+      </c>
+      <c r="G128" t="s">
+        <v>187</v>
+      </c>
+      <c r="I128" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>1777402020</v>
+      </c>
+      <c r="B129" t="s">
+        <v>9</v>
+      </c>
+      <c r="C129" t="s">
+        <v>153</v>
+      </c>
+      <c r="D129" t="s">
+        <v>203</v>
+      </c>
+      <c r="E129" t="s">
+        <v>177</v>
+      </c>
+      <c r="F129" t="s">
+        <v>179</v>
+      </c>
+      <c r="H129" t="s">
+        <v>187</v>
+      </c>
+      <c r="I129" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>1777402020</v>
+      </c>
+      <c r="B130" t="s">
+        <v>9</v>
+      </c>
+      <c r="C130" t="s">
+        <v>153</v>
+      </c>
+      <c r="D130" t="s">
+        <v>205</v>
+      </c>
+      <c r="E130" t="s">
+        <v>177</v>
+      </c>
+      <c r="F130" t="s">
+        <v>153</v>
+      </c>
+      <c r="G130" t="s">
+        <v>187</v>
+      </c>
+      <c r="I130" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>1777402020</v>
+      </c>
+      <c r="B131" t="s">
+        <v>9</v>
+      </c>
+      <c r="C131" t="s">
+        <v>153</v>
+      </c>
+      <c r="D131" t="s">
+        <v>205</v>
+      </c>
+      <c r="E131" t="s">
+        <v>177</v>
+      </c>
+      <c r="F131" t="s">
+        <v>179</v>
+      </c>
+      <c r="H131" t="s">
+        <v>187</v>
+      </c>
+      <c r="I131" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>1777402020</v>
+      </c>
+      <c r="B132" t="s">
+        <v>9</v>
+      </c>
+      <c r="C132" t="s">
+        <v>153</v>
+      </c>
+      <c r="D132" t="s">
+        <v>207</v>
+      </c>
+      <c r="E132" t="s">
+        <v>177</v>
+      </c>
+      <c r="F132" t="s">
+        <v>153</v>
+      </c>
+      <c r="G132" t="s">
+        <v>208</v>
+      </c>
+      <c r="I132" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>1777402020</v>
+      </c>
+      <c r="B133" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133" t="s">
+        <v>153</v>
+      </c>
+      <c r="D133" t="s">
+        <v>207</v>
+      </c>
+      <c r="E133" t="s">
+        <v>177</v>
+      </c>
+      <c r="F133" t="s">
+        <v>179</v>
+      </c>
+      <c r="H133" t="s">
+        <v>208</v>
+      </c>
+      <c r="I133" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>1777402020</v>
+      </c>
+      <c r="B134" t="s">
+        <v>9</v>
+      </c>
+      <c r="C134" t="s">
+        <v>153</v>
+      </c>
+      <c r="D134" t="s">
+        <v>210</v>
+      </c>
+      <c r="E134" t="s">
+        <v>177</v>
+      </c>
+      <c r="F134" t="s">
+        <v>153</v>
+      </c>
+      <c r="G134" t="s">
+        <v>36</v>
+      </c>
+      <c r="I134" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>1777402020</v>
+      </c>
+      <c r="B135" t="s">
+        <v>9</v>
+      </c>
+      <c r="C135" t="s">
+        <v>153</v>
+      </c>
+      <c r="D135" t="s">
+        <v>210</v>
+      </c>
+      <c r="E135" t="s">
+        <v>177</v>
+      </c>
+      <c r="F135" t="s">
+        <v>179</v>
+      </c>
+      <c r="H135" t="s">
+        <v>36</v>
+      </c>
+      <c r="I135" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>1777402020</v>
+      </c>
+      <c r="B136" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" t="s">
+        <v>153</v>
+      </c>
+      <c r="D136" t="s">
+        <v>212</v>
+      </c>
+      <c r="E136" t="s">
+        <v>213</v>
+      </c>
+      <c r="F136" t="s">
+        <v>153</v>
+      </c>
+      <c r="G136" t="s">
+        <v>214</v>
+      </c>
+      <c r="I136" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>1777402020</v>
+      </c>
+      <c r="B137" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137" t="s">
+        <v>153</v>
+      </c>
+      <c r="D137" t="s">
+        <v>212</v>
+      </c>
+      <c r="E137" t="s">
+        <v>213</v>
+      </c>
+      <c r="F137" t="s">
+        <v>179</v>
+      </c>
+      <c r="H137" t="s">
+        <v>214</v>
+      </c>
+      <c r="I137" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>1777402020</v>
+      </c>
+      <c r="B138" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" t="s">
+        <v>153</v>
+      </c>
+      <c r="D138" t="s">
+        <v>216</v>
+      </c>
+      <c r="E138" t="s">
+        <v>213</v>
+      </c>
+      <c r="F138" t="s">
+        <v>153</v>
+      </c>
+      <c r="G138" t="s">
+        <v>125</v>
+      </c>
+      <c r="I138" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <v>1777402020</v>
+      </c>
+      <c r="B139" t="s">
+        <v>9</v>
+      </c>
+      <c r="C139" t="s">
+        <v>153</v>
+      </c>
+      <c r="D139" t="s">
+        <v>216</v>
+      </c>
+      <c r="E139" t="s">
+        <v>213</v>
+      </c>
+      <c r="F139" t="s">
+        <v>179</v>
+      </c>
+      <c r="H139" t="s">
+        <v>125</v>
+      </c>
+      <c r="I139" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>1777402020</v>
+      </c>
+      <c r="B140" t="s">
+        <v>9</v>
+      </c>
+      <c r="C140" t="s">
+        <v>153</v>
+      </c>
+      <c r="D140" t="s">
+        <v>218</v>
+      </c>
+      <c r="E140" t="s">
+        <v>213</v>
+      </c>
+      <c r="F140" t="s">
+        <v>153</v>
+      </c>
+      <c r="G140" t="s">
+        <v>219</v>
+      </c>
+      <c r="I140" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>1777402020</v>
+      </c>
+      <c r="B141" t="s">
+        <v>9</v>
+      </c>
+      <c r="C141" t="s">
+        <v>153</v>
+      </c>
+      <c r="D141" t="s">
+        <v>218</v>
+      </c>
+      <c r="E141" t="s">
+        <v>213</v>
+      </c>
+      <c r="F141" t="s">
+        <v>179</v>
+      </c>
+      <c r="H141" t="s">
+        <v>219</v>
+      </c>
+      <c r="I141" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>1777402020</v>
+      </c>
+      <c r="B142" t="s">
+        <v>9</v>
+      </c>
+      <c r="C142" t="s">
+        <v>153</v>
+      </c>
+      <c r="D142" t="s">
+        <v>221</v>
+      </c>
+      <c r="E142" t="s">
+        <v>213</v>
+      </c>
+      <c r="F142" t="s">
+        <v>153</v>
+      </c>
+      <c r="G142" t="s">
+        <v>222</v>
+      </c>
+      <c r="I142" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <v>1777402020</v>
+      </c>
+      <c r="B143" t="s">
+        <v>9</v>
+      </c>
+      <c r="C143" t="s">
+        <v>153</v>
+      </c>
+      <c r="D143" t="s">
+        <v>221</v>
+      </c>
+      <c r="E143" t="s">
+        <v>213</v>
+      </c>
+      <c r="F143" t="s">
+        <v>179</v>
+      </c>
+      <c r="H143" t="s">
+        <v>222</v>
+      </c>
+      <c r="I143" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <v>1777402020</v>
+      </c>
+      <c r="B144" t="s">
+        <v>9</v>
+      </c>
+      <c r="C144" t="s">
+        <v>153</v>
+      </c>
+      <c r="D144" t="s">
+        <v>154</v>
+      </c>
+      <c r="E144" t="s">
+        <v>155</v>
+      </c>
+      <c r="F144" t="s">
+        <v>153</v>
+      </c>
+      <c r="G144" t="s">
+        <v>224</v>
+      </c>
+      <c r="I144" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>1777402020</v>
+      </c>
+      <c r="B145" t="s">
+        <v>9</v>
+      </c>
+      <c r="C145" t="s">
+        <v>153</v>
+      </c>
+      <c r="D145" t="s">
+        <v>154</v>
+      </c>
+      <c r="E145" t="s">
+        <v>155</v>
+      </c>
+      <c r="F145" t="s">
+        <v>179</v>
+      </c>
+      <c r="H145" t="s">
+        <v>224</v>
+      </c>
+      <c r="I145" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>1777402020</v>
+      </c>
+      <c r="B146" t="s">
+        <v>9</v>
+      </c>
+      <c r="C146" t="s">
+        <v>153</v>
+      </c>
+      <c r="D146" t="s">
+        <v>157</v>
+      </c>
+      <c r="E146" t="s">
+        <v>155</v>
+      </c>
+      <c r="F146" t="s">
+        <v>153</v>
+      </c>
+      <c r="G146" t="s">
+        <v>225</v>
+      </c>
+      <c r="I146" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>1777402020</v>
+      </c>
+      <c r="B147" t="s">
+        <v>9</v>
+      </c>
+      <c r="C147" t="s">
+        <v>153</v>
+      </c>
+      <c r="D147" t="s">
+        <v>157</v>
+      </c>
+      <c r="E147" t="s">
+        <v>155</v>
+      </c>
+      <c r="F147" t="s">
+        <v>179</v>
+      </c>
+      <c r="H147" t="s">
+        <v>225</v>
+      </c>
+      <c r="I147" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>1777402020</v>
+      </c>
+      <c r="B148" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" t="s">
+        <v>153</v>
+      </c>
+      <c r="D148" t="s">
+        <v>159</v>
+      </c>
+      <c r="E148" t="s">
+        <v>155</v>
+      </c>
+      <c r="F148" t="s">
+        <v>153</v>
+      </c>
+      <c r="G148" t="s">
+        <v>125</v>
+      </c>
+      <c r="I148" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>1777402020</v>
+      </c>
+      <c r="B149" t="s">
+        <v>9</v>
+      </c>
+      <c r="C149" t="s">
+        <v>153</v>
+      </c>
+      <c r="D149" t="s">
+        <v>159</v>
+      </c>
+      <c r="E149" t="s">
+        <v>155</v>
+      </c>
+      <c r="F149" t="s">
+        <v>179</v>
+      </c>
+      <c r="H149" t="s">
+        <v>125</v>
+      </c>
+      <c r="I149" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>1777402020</v>
+      </c>
+      <c r="B150" t="s">
+        <v>9</v>
+      </c>
+      <c r="C150" t="s">
+        <v>153</v>
+      </c>
+      <c r="D150" t="s">
+        <v>162</v>
+      </c>
+      <c r="E150" t="s">
+        <v>155</v>
+      </c>
+      <c r="F150" t="s">
+        <v>153</v>
+      </c>
+      <c r="G150" t="s">
+        <v>226</v>
+      </c>
+      <c r="I150" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>1777402020</v>
+      </c>
+      <c r="B151" t="s">
+        <v>9</v>
+      </c>
+      <c r="C151" t="s">
+        <v>153</v>
+      </c>
+      <c r="D151" t="s">
+        <v>162</v>
+      </c>
+      <c r="E151" t="s">
+        <v>155</v>
+      </c>
+      <c r="F151" t="s">
+        <v>179</v>
+      </c>
+      <c r="H151" t="s">
+        <v>226</v>
+      </c>
+      <c r="I151" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>1777402020</v>
+      </c>
+      <c r="B152" t="s">
+        <v>9</v>
+      </c>
+      <c r="C152" t="s">
+        <v>153</v>
+      </c>
+      <c r="D152" t="s">
+        <v>166</v>
+      </c>
+      <c r="E152" t="s">
+        <v>155</v>
+      </c>
+      <c r="F152" t="s">
+        <v>153</v>
+      </c>
+      <c r="G152" t="s">
+        <v>111</v>
+      </c>
+      <c r="I152" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>1777402020</v>
+      </c>
+      <c r="B153" t="s">
+        <v>9</v>
+      </c>
+      <c r="C153" t="s">
+        <v>153</v>
+      </c>
+      <c r="D153" t="s">
+        <v>166</v>
+      </c>
+      <c r="E153" t="s">
+        <v>155</v>
+      </c>
+      <c r="F153" t="s">
+        <v>179</v>
+      </c>
+      <c r="H153" t="s">
+        <v>111</v>
+      </c>
+      <c r="I153" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>1777402730</v>
+      </c>
+      <c r="B154" t="s">
+        <v>9</v>
+      </c>
+      <c r="C154" t="s">
+        <v>153</v>
+      </c>
+      <c r="D154" t="s">
+        <v>166</v>
+      </c>
+      <c r="E154" t="s">
+        <v>155</v>
+      </c>
+      <c r="F154" t="s">
+        <v>153</v>
+      </c>
+      <c r="G154" t="s">
+        <v>111</v>
+      </c>
+      <c r="H154" t="s">
+        <v>227</v>
+      </c>
+      <c r="I154" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update: demo data tu have evolution timestamp in the futur
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1172,6 +1172,72 @@
   </si>
   <si>
     <t>Liste des 3 principales langues suisses et leurs sigles</t>
+  </si>
+  <si>
+    <t>01-pop</t>
+  </si>
+  <si>
+    <t>2028/03</t>
+  </si>
+  <si>
+    <t>02-espace</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>2028</t>
+  </si>
+  <si>
+    <t>last_update_date</t>
+  </si>
+  <si>
+    <t>2020/03/25</t>
+  </si>
+  <si>
+    <t>2026/03/25</t>
+  </si>
+  <si>
+    <t>06-industrie</t>
+  </si>
+  <si>
+    <t>2023/09</t>
+  </si>
+  <si>
+    <t>2029/09</t>
+  </si>
+  <si>
+    <t>2011/03/02</t>
+  </si>
+  <si>
+    <t>2026/04/25</t>
+  </si>
+  <si>
+    <t>14-sante</t>
+  </si>
+  <si>
+    <t>2026/04/20</t>
+  </si>
+  <si>
+    <t>poste</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>2030</t>
+  </si>
+  <si>
+    <t>2018/08</t>
+  </si>
+  <si>
+    <t>2028/08</t>
+  </si>
+  <si>
+    <t>ofs-sys-form</t>
+  </si>
+  <si>
+    <t>2029/10</t>
   </si>
 </sst>
 </file>
@@ -9267,6 +9333,207 @@
         <v>385</v>
       </c>
     </row>
+    <row r="364">
+      <c r="A364">
+        <v>1777490030</v>
+      </c>
+      <c r="B364" t="s">
+        <v>9</v>
+      </c>
+      <c r="C364" t="s">
+        <v>84</v>
+      </c>
+      <c r="D364" t="s">
+        <v>386</v>
+      </c>
+      <c r="F364" t="s">
+        <v>18</v>
+      </c>
+      <c r="H364" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365">
+        <v>1777490030</v>
+      </c>
+      <c r="B365" t="s">
+        <v>9</v>
+      </c>
+      <c r="C365" t="s">
+        <v>84</v>
+      </c>
+      <c r="D365" t="s">
+        <v>388</v>
+      </c>
+      <c r="F365" t="s">
+        <v>18</v>
+      </c>
+      <c r="G365" t="s">
+        <v>389</v>
+      </c>
+      <c r="H365" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366">
+        <v>1777490030</v>
+      </c>
+      <c r="B366" t="s">
+        <v>9</v>
+      </c>
+      <c r="C366" t="s">
+        <v>84</v>
+      </c>
+      <c r="D366" t="s">
+        <v>388</v>
+      </c>
+      <c r="F366" t="s">
+        <v>391</v>
+      </c>
+      <c r="G366" t="s">
+        <v>392</v>
+      </c>
+      <c r="H366" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367">
+        <v>1777490030</v>
+      </c>
+      <c r="B367" t="s">
+        <v>9</v>
+      </c>
+      <c r="C367" t="s">
+        <v>84</v>
+      </c>
+      <c r="D367" t="s">
+        <v>394</v>
+      </c>
+      <c r="F367" t="s">
+        <v>18</v>
+      </c>
+      <c r="G367" t="s">
+        <v>395</v>
+      </c>
+      <c r="H367" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368">
+        <v>1777490030</v>
+      </c>
+      <c r="B368" t="s">
+        <v>9</v>
+      </c>
+      <c r="C368" t="s">
+        <v>84</v>
+      </c>
+      <c r="D368" t="s">
+        <v>85</v>
+      </c>
+      <c r="F368" t="s">
+        <v>391</v>
+      </c>
+      <c r="G368" t="s">
+        <v>397</v>
+      </c>
+      <c r="H368" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369">
+        <v>1777490030</v>
+      </c>
+      <c r="B369" t="s">
+        <v>9</v>
+      </c>
+      <c r="C369" t="s">
+        <v>84</v>
+      </c>
+      <c r="D369" t="s">
+        <v>399</v>
+      </c>
+      <c r="F369" t="s">
+        <v>391</v>
+      </c>
+      <c r="H369" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370">
+        <v>1777490074</v>
+      </c>
+      <c r="B370" t="s">
+        <v>9</v>
+      </c>
+      <c r="C370" t="s">
+        <v>56</v>
+      </c>
+      <c r="D370" t="s">
+        <v>401</v>
+      </c>
+      <c r="F370" t="s">
+        <v>18</v>
+      </c>
+      <c r="G370" t="s">
+        <v>402</v>
+      </c>
+      <c r="H370" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371">
+        <v>1777490074</v>
+      </c>
+      <c r="B371" t="s">
+        <v>9</v>
+      </c>
+      <c r="C371" t="s">
+        <v>56</v>
+      </c>
+      <c r="D371" t="s">
+        <v>57</v>
+      </c>
+      <c r="F371" t="s">
+        <v>18</v>
+      </c>
+      <c r="G371" t="s">
+        <v>404</v>
+      </c>
+      <c r="H371" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372">
+        <v>1777490074</v>
+      </c>
+      <c r="B372" t="s">
+        <v>9</v>
+      </c>
+      <c r="C372" t="s">
+        <v>56</v>
+      </c>
+      <c r="D372" t="s">
+        <v>406</v>
+      </c>
+      <c r="F372" t="s">
+        <v>18</v>
+      </c>
+      <c r="G372" t="s">
+        <v>389</v>
+      </c>
+      <c r="H372" t="s">
+        <v>407</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change: evolution tables now open around the current date, at the boundary between future and past entries (#127)
* fix: adjust margin for freq-percent class in Datatable.svelte

* update: demo data tu have evolution timestamp in the futur

* Open evolution tables around current date
</commit_message>
<xml_diff>
--- a/public/data/db-source/evolution.xlsx
+++ b/public/data/db-source/evolution.xlsx
@@ -1172,6 +1172,72 @@
   </si>
   <si>
     <t>Liste des 3 principales langues suisses et leurs sigles</t>
+  </si>
+  <si>
+    <t>01-pop</t>
+  </si>
+  <si>
+    <t>2028/03</t>
+  </si>
+  <si>
+    <t>02-espace</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>2028</t>
+  </si>
+  <si>
+    <t>last_update_date</t>
+  </si>
+  <si>
+    <t>2020/03/25</t>
+  </si>
+  <si>
+    <t>2026/03/25</t>
+  </si>
+  <si>
+    <t>06-industrie</t>
+  </si>
+  <si>
+    <t>2023/09</t>
+  </si>
+  <si>
+    <t>2029/09</t>
+  </si>
+  <si>
+    <t>2011/03/02</t>
+  </si>
+  <si>
+    <t>2026/04/25</t>
+  </si>
+  <si>
+    <t>14-sante</t>
+  </si>
+  <si>
+    <t>2026/04/20</t>
+  </si>
+  <si>
+    <t>poste</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>2030</t>
+  </si>
+  <si>
+    <t>2018/08</t>
+  </si>
+  <si>
+    <t>2028/08</t>
+  </si>
+  <si>
+    <t>ofs-sys-form</t>
+  </si>
+  <si>
+    <t>2029/10</t>
   </si>
 </sst>
 </file>
@@ -9267,6 +9333,207 @@
         <v>385</v>
       </c>
     </row>
+    <row r="364">
+      <c r="A364">
+        <v>1777490030</v>
+      </c>
+      <c r="B364" t="s">
+        <v>9</v>
+      </c>
+      <c r="C364" t="s">
+        <v>84</v>
+      </c>
+      <c r="D364" t="s">
+        <v>386</v>
+      </c>
+      <c r="F364" t="s">
+        <v>18</v>
+      </c>
+      <c r="H364" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365">
+        <v>1777490030</v>
+      </c>
+      <c r="B365" t="s">
+        <v>9</v>
+      </c>
+      <c r="C365" t="s">
+        <v>84</v>
+      </c>
+      <c r="D365" t="s">
+        <v>388</v>
+      </c>
+      <c r="F365" t="s">
+        <v>18</v>
+      </c>
+      <c r="G365" t="s">
+        <v>389</v>
+      </c>
+      <c r="H365" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366">
+        <v>1777490030</v>
+      </c>
+      <c r="B366" t="s">
+        <v>9</v>
+      </c>
+      <c r="C366" t="s">
+        <v>84</v>
+      </c>
+      <c r="D366" t="s">
+        <v>388</v>
+      </c>
+      <c r="F366" t="s">
+        <v>391</v>
+      </c>
+      <c r="G366" t="s">
+        <v>392</v>
+      </c>
+      <c r="H366" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367">
+        <v>1777490030</v>
+      </c>
+      <c r="B367" t="s">
+        <v>9</v>
+      </c>
+      <c r="C367" t="s">
+        <v>84</v>
+      </c>
+      <c r="D367" t="s">
+        <v>394</v>
+      </c>
+      <c r="F367" t="s">
+        <v>18</v>
+      </c>
+      <c r="G367" t="s">
+        <v>395</v>
+      </c>
+      <c r="H367" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368">
+        <v>1777490030</v>
+      </c>
+      <c r="B368" t="s">
+        <v>9</v>
+      </c>
+      <c r="C368" t="s">
+        <v>84</v>
+      </c>
+      <c r="D368" t="s">
+        <v>85</v>
+      </c>
+      <c r="F368" t="s">
+        <v>391</v>
+      </c>
+      <c r="G368" t="s">
+        <v>397</v>
+      </c>
+      <c r="H368" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369">
+        <v>1777490030</v>
+      </c>
+      <c r="B369" t="s">
+        <v>9</v>
+      </c>
+      <c r="C369" t="s">
+        <v>84</v>
+      </c>
+      <c r="D369" t="s">
+        <v>399</v>
+      </c>
+      <c r="F369" t="s">
+        <v>391</v>
+      </c>
+      <c r="H369" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370">
+        <v>1777490074</v>
+      </c>
+      <c r="B370" t="s">
+        <v>9</v>
+      </c>
+      <c r="C370" t="s">
+        <v>56</v>
+      </c>
+      <c r="D370" t="s">
+        <v>401</v>
+      </c>
+      <c r="F370" t="s">
+        <v>18</v>
+      </c>
+      <c r="G370" t="s">
+        <v>402</v>
+      </c>
+      <c r="H370" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371">
+        <v>1777490074</v>
+      </c>
+      <c r="B371" t="s">
+        <v>9</v>
+      </c>
+      <c r="C371" t="s">
+        <v>56</v>
+      </c>
+      <c r="D371" t="s">
+        <v>57</v>
+      </c>
+      <c r="F371" t="s">
+        <v>18</v>
+      </c>
+      <c r="G371" t="s">
+        <v>404</v>
+      </c>
+      <c r="H371" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372">
+        <v>1777490074</v>
+      </c>
+      <c r="B372" t="s">
+        <v>9</v>
+      </c>
+      <c r="C372" t="s">
+        <v>56</v>
+      </c>
+      <c r="D372" t="s">
+        <v>406</v>
+      </c>
+      <c r="F372" t="s">
+        <v>18</v>
+      </c>
+      <c r="G372" t="s">
+        <v>389</v>
+      </c>
+      <c r="H372" t="s">
+        <v>407</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>